<commit_message>
Refine clean sheet player stats
</commit_message>
<xml_diff>
--- a/data/生康足球队数据源.xlsx
+++ b/data/生康足球队数据源.xlsx
@@ -13,7 +13,7 @@
     <sheet name="赛程" sheetId="4" r:id="rId4"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">球员数据!$A$1:$O$18</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">球员数据!$A$1:$N$18</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">赛事索引!$A$1:$F$4</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">赛程!$A$1:$I$12</definedName>
   </definedNames>
@@ -35,7 +35,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="245" uniqueCount="172">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="244" uniqueCount="171">
   <si>
     <t>生康足球队 · 球员数据汇总</t>
   </si>
@@ -104,9 +104,6 @@
   </si>
   <si>
     <t>MVP</t>
-  </si>
-  <si>
-    <t>扑救</t>
   </si>
   <si>
     <t>零封</t>
@@ -1721,7 +1718,7 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
-  <dimension ref="A1:O18"/>
+  <dimension ref="A1:N18"/>
   <sheetFormatPr defaultColWidth="9" defaultRowHeight="13.5"/>
   <cols>
     <col min="1" max="1" width="8" customWidth="1"/>
@@ -1730,13 +1727,13 @@
     <col min="4" max="4" width="8" customWidth="1"/>
     <col min="5" max="5" width="10" customWidth="1"/>
     <col min="6" max="6" width="17" customWidth="1"/>
-    <col min="7" max="12" width="9" customWidth="1"/>
-    <col min="13" max="13" width="12" customWidth="1"/>
-    <col min="14" max="14" width="20" customWidth="1"/>
-    <col min="15" max="15" width="28" customWidth="1"/>
+    <col min="7" max="11" width="9" customWidth="1"/>
+    <col min="12" max="12" width="12" customWidth="1"/>
+    <col min="13" max="13" width="20" customWidth="1"/>
+    <col min="14" max="15" width="28" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" ht="26" customHeight="1" spans="1:15">
+    <row r="1" ht="26" customHeight="1" spans="1:14">
       <c r="A1" s="4" t="s">
         <v>13</v>
       </c>
@@ -1779,28 +1776,25 @@
       <c r="N1" s="4" t="s">
         <v>26</v>
       </c>
-      <c r="O1" s="4" t="s">
-        <v>27</v>
-      </c>
-    </row>
-    <row r="2" ht="23" customHeight="1" spans="1:15">
+    </row>
+    <row r="2" ht="23" customHeight="1" spans="1:14">
       <c r="A2" s="2">
         <v>1</v>
       </c>
       <c r="B2" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="C2" s="2" t="s">
         <v>28</v>
-      </c>
-      <c r="C2" s="2" t="s">
-        <v>29</v>
       </c>
       <c r="D2" s="2">
         <v>6</v>
       </c>
       <c r="E2" s="2" t="s">
+        <v>29</v>
+      </c>
+      <c r="F2" s="2" t="s">
         <v>30</v>
-      </c>
-      <c r="F2" s="2" t="s">
-        <v>31</v>
       </c>
       <c r="G2" s="2">
         <v>11</v>
@@ -1817,39 +1811,36 @@
       <c r="K2" s="2">
         <v>0</v>
       </c>
-      <c r="L2" s="2">
-        <v>0</v>
-      </c>
-      <c r="M2" s="5">
-        <f t="shared" ref="M2:M18" si="0">ROUND(MIN(9.5,MAX(6,6+G2*0.08+H2*0.35+I2*0.25+J2*0.25+K2*0.03+L2*0.15)),1)</f>
+      <c r="L2" s="5">
+        <f t="shared" ref="L2:L18" si="0">ROUND(MIN(9.5,MAX(6,6+G2*0.08+H2*0.35+I2*0.25+J2*0.25+K2*0.15)),1)</f>
         <v>7.1</v>
       </c>
-      <c r="N2" s="2" t="s">
-        <v>32</v>
-      </c>
-      <c r="O2" s="2" t="str">
-        <f t="shared" ref="O2:O18" si="1">IF(H2&gt;0,IF(I2&gt;0,"贡献 "&amp;H2&amp;" 粒进球 / 送出 "&amp;I2&amp;" 次助攻","贡献 "&amp;H2&amp;" 粒进球"),IF(I2&gt;0,"送出 "&amp;I2&amp;" 次助攻","累计出场 "&amp;G2&amp;" 场"))</f>
+      <c r="M2" s="2" t="s">
+        <v>31</v>
+      </c>
+      <c r="N2" s="2" t="str">
+        <f t="shared" ref="N2:N18" si="1">IF(H2&gt;0,IF(I2&gt;0,"贡献 "&amp;H2&amp;" 粒进球 / 送出 "&amp;I2&amp;" 次助攻","贡献 "&amp;H2&amp;" 粒进球"),IF(I2&gt;0,"送出 "&amp;I2&amp;" 次助攻","累计出场 "&amp;G2&amp;" 场"))</f>
         <v>送出 1 次助攻</v>
       </c>
     </row>
-    <row r="3" ht="23" customHeight="1" spans="1:15">
+    <row r="3" ht="23" customHeight="1" spans="1:14">
       <c r="A3" s="3">
         <v>2</v>
       </c>
       <c r="B3" s="3" t="s">
+        <v>32</v>
+      </c>
+      <c r="C3" s="3" t="s">
         <v>33</v>
-      </c>
-      <c r="C3" s="3" t="s">
-        <v>34</v>
       </c>
       <c r="D3" s="3">
         <v>10</v>
       </c>
       <c r="E3" s="3" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="F3" s="3" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="G3" s="3">
         <v>4</v>
@@ -1866,39 +1857,36 @@
       <c r="K3" s="3">
         <v>0</v>
       </c>
-      <c r="L3" s="3">
-        <v>0</v>
-      </c>
-      <c r="M3" s="6">
+      <c r="L3" s="6">
         <f t="shared" si="0"/>
         <v>6.3</v>
       </c>
-      <c r="N3" s="3" t="s">
-        <v>36</v>
-      </c>
-      <c r="O3" s="3" t="str">
+      <c r="M3" s="3" t="s">
+        <v>35</v>
+      </c>
+      <c r="N3" s="3" t="str">
         <f t="shared" si="1"/>
         <v>累计出场 4 场</v>
       </c>
     </row>
-    <row r="4" ht="23" customHeight="1" spans="1:15">
+    <row r="4" ht="23" customHeight="1" spans="1:14">
       <c r="A4" s="2">
         <v>3</v>
       </c>
       <c r="B4" s="2" t="s">
+        <v>36</v>
+      </c>
+      <c r="C4" s="2" t="s">
         <v>37</v>
-      </c>
-      <c r="C4" s="2" t="s">
-        <v>38</v>
       </c>
       <c r="D4" s="2">
         <v>29</v>
       </c>
       <c r="E4" s="2" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="F4" s="2" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="G4" s="2">
         <v>9</v>
@@ -1915,39 +1903,36 @@
       <c r="K4" s="2">
         <v>0</v>
       </c>
-      <c r="L4" s="2">
-        <v>0</v>
-      </c>
-      <c r="M4" s="5">
+      <c r="L4" s="5">
         <f t="shared" si="0"/>
         <v>6.7</v>
       </c>
-      <c r="N4" s="2" t="s">
-        <v>40</v>
-      </c>
-      <c r="O4" s="2" t="str">
+      <c r="M4" s="2" t="s">
+        <v>39</v>
+      </c>
+      <c r="N4" s="2" t="str">
         <f t="shared" si="1"/>
         <v>累计出场 9 场</v>
       </c>
     </row>
-    <row r="5" ht="23" customHeight="1" spans="1:15">
+    <row r="5" ht="23" customHeight="1" spans="1:14">
       <c r="A5" s="3">
         <v>4</v>
       </c>
       <c r="B5" s="3" t="s">
+        <v>40</v>
+      </c>
+      <c r="C5" s="3" t="s">
         <v>41</v>
       </c>
-      <c r="C5" s="3" t="s">
+      <c r="D5" s="3">
+        <v>0</v>
+      </c>
+      <c r="E5" s="3" t="s">
         <v>42</v>
       </c>
-      <c r="D5" s="3">
-        <v>0</v>
-      </c>
-      <c r="E5" s="3" t="s">
-        <v>43</v>
-      </c>
       <c r="F5" s="3" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="G5" s="3">
         <v>8</v>
@@ -1962,41 +1947,38 @@
         <v>0</v>
       </c>
       <c r="K5" s="3">
-        <v>0</v>
-      </c>
-      <c r="L5" s="3">
         <v>1</v>
       </c>
-      <c r="M5" s="6">
+      <c r="L5" s="6">
         <f t="shared" si="0"/>
         <v>6.8</v>
       </c>
-      <c r="N5" s="3" t="s">
-        <v>44</v>
-      </c>
-      <c r="O5" s="3" t="str">
+      <c r="M5" s="3" t="s">
+        <v>43</v>
+      </c>
+      <c r="N5" s="3" t="str">
         <f t="shared" si="1"/>
         <v>累计出场 8 场</v>
       </c>
     </row>
-    <row r="6" ht="23" customHeight="1" spans="1:15">
+    <row r="6" ht="23" customHeight="1" spans="1:14">
       <c r="A6" s="2">
         <v>5</v>
       </c>
       <c r="B6" s="2" t="s">
+        <v>44</v>
+      </c>
+      <c r="C6" s="2" t="s">
         <v>45</v>
-      </c>
-      <c r="C6" s="2" t="s">
-        <v>46</v>
       </c>
       <c r="D6" s="2">
         <v>23</v>
       </c>
       <c r="E6" s="2" t="s">
+        <v>46</v>
+      </c>
+      <c r="F6" s="2" t="s">
         <v>47</v>
-      </c>
-      <c r="F6" s="2" t="s">
-        <v>48</v>
       </c>
       <c r="G6" s="2">
         <v>8</v>
@@ -2013,39 +1995,36 @@
       <c r="K6" s="2">
         <v>0</v>
       </c>
-      <c r="L6" s="2">
-        <v>0</v>
-      </c>
-      <c r="M6" s="5">
+      <c r="L6" s="5">
         <f t="shared" si="0"/>
         <v>6.6</v>
       </c>
-      <c r="N6" s="2" t="s">
-        <v>49</v>
-      </c>
-      <c r="O6" s="2" t="str">
+      <c r="M6" s="2" t="s">
+        <v>48</v>
+      </c>
+      <c r="N6" s="2" t="str">
         <f t="shared" si="1"/>
         <v>累计出场 8 场</v>
       </c>
     </row>
-    <row r="7" ht="23" customHeight="1" spans="1:15">
+    <row r="7" ht="23" customHeight="1" spans="1:14">
       <c r="A7" s="3">
         <v>6</v>
       </c>
       <c r="B7" s="3" t="s">
+        <v>49</v>
+      </c>
+      <c r="C7" s="3" t="s">
         <v>50</v>
-      </c>
-      <c r="C7" s="3" t="s">
-        <v>51</v>
       </c>
       <c r="D7" s="3">
         <v>9</v>
       </c>
       <c r="E7" s="3" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="F7" s="3" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="G7" s="3">
         <v>0</v>
@@ -2062,39 +2041,36 @@
       <c r="K7" s="3">
         <v>0</v>
       </c>
-      <c r="L7" s="3">
-        <v>0</v>
-      </c>
-      <c r="M7" s="6">
+      <c r="L7" s="6">
         <f t="shared" si="0"/>
         <v>6</v>
       </c>
-      <c r="N7" s="3" t="s">
-        <v>53</v>
-      </c>
-      <c r="O7" s="3" t="str">
+      <c r="M7" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="N7" s="3" t="str">
         <f t="shared" si="1"/>
         <v>累计出场 0 场</v>
       </c>
     </row>
-    <row r="8" ht="23" customHeight="1" spans="1:15">
+    <row r="8" ht="23" customHeight="1" spans="1:14">
       <c r="A8" s="2">
         <v>7</v>
       </c>
       <c r="B8" s="2" t="s">
+        <v>53</v>
+      </c>
+      <c r="C8" s="2" t="s">
         <v>54</v>
-      </c>
-      <c r="C8" s="2" t="s">
-        <v>55</v>
       </c>
       <c r="D8" s="2">
         <v>15</v>
       </c>
       <c r="E8" s="2" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="F8" s="2" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="G8" s="2">
         <v>11</v>
@@ -2111,39 +2087,36 @@
       <c r="K8" s="2">
         <v>0</v>
       </c>
-      <c r="L8" s="2">
-        <v>0</v>
-      </c>
-      <c r="M8" s="5">
+      <c r="L8" s="5">
         <f t="shared" si="0"/>
         <v>9.2</v>
       </c>
-      <c r="N8" s="2" t="s">
-        <v>57</v>
-      </c>
-      <c r="O8" s="2" t="str">
+      <c r="M8" s="2" t="s">
+        <v>56</v>
+      </c>
+      <c r="N8" s="2" t="str">
         <f t="shared" si="1"/>
         <v>贡献 6 粒进球 / 送出 1 次助攻</v>
       </c>
     </row>
-    <row r="9" ht="23" customHeight="1" spans="1:15">
+    <row r="9" ht="23" customHeight="1" spans="1:14">
       <c r="A9" s="3">
         <v>8</v>
       </c>
       <c r="B9" s="3" t="s">
+        <v>57</v>
+      </c>
+      <c r="C9" s="3" t="s">
         <v>58</v>
-      </c>
-      <c r="C9" s="3" t="s">
-        <v>59</v>
       </c>
       <c r="D9" s="3">
         <v>8</v>
       </c>
       <c r="E9" s="3" t="s">
+        <v>59</v>
+      </c>
+      <c r="F9" s="3" t="s">
         <v>60</v>
-      </c>
-      <c r="F9" s="3" t="s">
-        <v>61</v>
       </c>
       <c r="G9" s="3">
         <v>8</v>
@@ -2160,39 +2133,36 @@
       <c r="K9" s="3">
         <v>0</v>
       </c>
-      <c r="L9" s="3">
-        <v>0</v>
-      </c>
-      <c r="M9" s="6">
+      <c r="L9" s="6">
         <f t="shared" si="0"/>
         <v>8.1</v>
       </c>
-      <c r="N9" s="3" t="s">
-        <v>62</v>
-      </c>
-      <c r="O9" s="3" t="str">
+      <c r="M9" s="3" t="s">
+        <v>61</v>
+      </c>
+      <c r="N9" s="3" t="str">
         <f t="shared" si="1"/>
         <v>贡献 2 粒进球 / 送出 3 次助攻</v>
       </c>
     </row>
-    <row r="10" ht="23" customHeight="1" spans="1:15">
+    <row r="10" ht="23" customHeight="1" spans="1:14">
       <c r="A10" s="2">
         <v>9</v>
       </c>
       <c r="B10" s="2" t="s">
+        <v>62</v>
+      </c>
+      <c r="C10" s="2" t="s">
         <v>63</v>
-      </c>
-      <c r="C10" s="2" t="s">
-        <v>64</v>
       </c>
       <c r="D10" s="2">
         <v>5</v>
       </c>
       <c r="E10" s="2" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="F10" s="2" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="G10" s="2">
         <v>10</v>
@@ -2209,39 +2179,36 @@
       <c r="K10" s="2">
         <v>0</v>
       </c>
-      <c r="L10" s="2">
-        <v>0</v>
-      </c>
-      <c r="M10" s="5">
+      <c r="L10" s="5">
         <f t="shared" si="0"/>
         <v>9</v>
       </c>
-      <c r="N10" s="2" t="s">
-        <v>66</v>
-      </c>
-      <c r="O10" s="2" t="str">
+      <c r="M10" s="2" t="s">
+        <v>65</v>
+      </c>
+      <c r="N10" s="2" t="str">
         <f t="shared" si="1"/>
         <v>贡献 4 粒进球 / 送出 3 次助攻</v>
       </c>
     </row>
-    <row r="11" ht="23" customHeight="1" spans="1:15">
+    <row r="11" ht="23" customHeight="1" spans="1:14">
       <c r="A11" s="3">
         <v>10</v>
       </c>
       <c r="B11" s="3" t="s">
+        <v>66</v>
+      </c>
+      <c r="C11" s="3" t="s">
         <v>67</v>
-      </c>
-      <c r="C11" s="3" t="s">
-        <v>68</v>
       </c>
       <c r="D11" s="3">
         <v>17</v>
       </c>
       <c r="E11" s="3" t="s">
+        <v>29</v>
+      </c>
+      <c r="F11" s="3" t="s">
         <v>30</v>
-      </c>
-      <c r="F11" s="3" t="s">
-        <v>31</v>
       </c>
       <c r="G11" s="3">
         <v>6</v>
@@ -2258,39 +2225,36 @@
       <c r="K11" s="3">
         <v>0</v>
       </c>
-      <c r="L11" s="3">
-        <v>0</v>
-      </c>
-      <c r="M11" s="6">
+      <c r="L11" s="6">
         <f t="shared" si="0"/>
         <v>6.5</v>
       </c>
-      <c r="N11" s="3" t="s">
-        <v>69</v>
-      </c>
-      <c r="O11" s="3" t="str">
+      <c r="M11" s="3" t="s">
+        <v>68</v>
+      </c>
+      <c r="N11" s="3" t="str">
         <f t="shared" si="1"/>
         <v>累计出场 6 场</v>
       </c>
     </row>
-    <row r="12" ht="23" customHeight="1" spans="1:15">
+    <row r="12" ht="23" customHeight="1" spans="1:14">
       <c r="A12" s="2">
         <v>11</v>
       </c>
       <c r="B12" s="2" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="C12" s="2" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="D12" s="2">
         <v>18</v>
       </c>
       <c r="E12" s="2" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="F12" s="2" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="G12" s="2">
         <v>5</v>
@@ -2305,41 +2269,38 @@
         <v>0</v>
       </c>
       <c r="K12" s="2">
-        <v>0</v>
-      </c>
-      <c r="L12" s="2">
         <v>1</v>
       </c>
-      <c r="M12" s="5">
+      <c r="L12" s="5">
         <f t="shared" si="0"/>
         <v>6.6</v>
       </c>
-      <c r="N12" s="2" t="s">
-        <v>44</v>
-      </c>
-      <c r="O12" s="2" t="str">
+      <c r="M12" s="2" t="s">
+        <v>43</v>
+      </c>
+      <c r="N12" s="2" t="str">
         <f t="shared" si="1"/>
         <v>累计出场 5 场</v>
       </c>
     </row>
-    <row r="13" ht="23" customHeight="1" spans="1:15">
+    <row r="13" ht="23" customHeight="1" spans="1:14">
       <c r="A13" s="3">
         <v>12</v>
       </c>
       <c r="B13" s="3" t="s">
+        <v>71</v>
+      </c>
+      <c r="C13" s="3" t="s">
         <v>72</v>
-      </c>
-      <c r="C13" s="3" t="s">
-        <v>73</v>
       </c>
       <c r="D13" s="3">
         <v>19</v>
       </c>
       <c r="E13" s="3" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="F13" s="3" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="G13" s="3">
         <v>8</v>
@@ -2356,39 +2317,36 @@
       <c r="K13" s="3">
         <v>0</v>
       </c>
-      <c r="L13" s="3">
-        <v>0</v>
-      </c>
-      <c r="M13" s="6">
+      <c r="L13" s="6">
         <f t="shared" si="0"/>
         <v>6.6</v>
       </c>
-      <c r="N13" s="3" t="s">
-        <v>74</v>
-      </c>
-      <c r="O13" s="3" t="str">
+      <c r="M13" s="3" t="s">
+        <v>73</v>
+      </c>
+      <c r="N13" s="3" t="str">
         <f t="shared" si="1"/>
         <v>累计出场 8 场</v>
       </c>
     </row>
-    <row r="14" ht="23" customHeight="1" spans="1:15">
+    <row r="14" ht="23" customHeight="1" spans="1:14">
       <c r="A14" s="2">
         <v>13</v>
       </c>
       <c r="B14" s="2" t="s">
+        <v>74</v>
+      </c>
+      <c r="C14" s="2" t="s">
         <v>75</v>
-      </c>
-      <c r="C14" s="2" t="s">
-        <v>76</v>
       </c>
       <c r="D14" s="2">
         <v>25</v>
       </c>
       <c r="E14" s="2" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="F14" s="2" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="G14" s="2">
         <v>6</v>
@@ -2405,39 +2363,36 @@
       <c r="K14" s="2">
         <v>0</v>
       </c>
-      <c r="L14" s="2">
-        <v>0</v>
-      </c>
-      <c r="M14" s="5">
+      <c r="L14" s="5">
         <f t="shared" si="0"/>
         <v>6.5</v>
       </c>
-      <c r="N14" s="2" t="s">
-        <v>69</v>
-      </c>
-      <c r="O14" s="2" t="str">
+      <c r="M14" s="2" t="s">
+        <v>68</v>
+      </c>
+      <c r="N14" s="2" t="str">
         <f t="shared" si="1"/>
         <v>累计出场 6 场</v>
       </c>
     </row>
-    <row r="15" ht="23" customHeight="1" spans="1:15">
+    <row r="15" ht="23" customHeight="1" spans="1:14">
       <c r="A15" s="3">
         <v>14</v>
       </c>
       <c r="B15" s="3" t="s">
+        <v>77</v>
+      </c>
+      <c r="C15" s="3" t="s">
         <v>78</v>
-      </c>
-      <c r="C15" s="3" t="s">
-        <v>79</v>
       </c>
       <c r="D15" s="3">
         <v>66</v>
       </c>
       <c r="E15" s="3" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="F15" s="3" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="G15" s="3">
         <v>3</v>
@@ -2454,39 +2409,36 @@
       <c r="K15" s="3">
         <v>0</v>
       </c>
-      <c r="L15" s="3">
-        <v>0</v>
-      </c>
-      <c r="M15" s="6">
+      <c r="L15" s="6">
         <f t="shared" si="0"/>
         <v>6.2</v>
       </c>
-      <c r="N15" s="3" t="s">
-        <v>53</v>
-      </c>
-      <c r="O15" s="3" t="str">
+      <c r="M15" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="N15" s="3" t="str">
         <f t="shared" si="1"/>
         <v>累计出场 3 场</v>
       </c>
     </row>
-    <row r="16" ht="23" customHeight="1" spans="1:15">
+    <row r="16" ht="23" customHeight="1" spans="1:14">
       <c r="A16" s="2">
         <v>15</v>
       </c>
       <c r="B16" s="2" t="s">
+        <v>80</v>
+      </c>
+      <c r="C16" s="2" t="s">
         <v>81</v>
-      </c>
-      <c r="C16" s="2" t="s">
-        <v>82</v>
       </c>
       <c r="D16" s="2">
         <v>12</v>
       </c>
       <c r="E16" s="2" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="F16" s="2" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="G16" s="2">
         <v>10</v>
@@ -2501,41 +2453,38 @@
         <v>0</v>
       </c>
       <c r="K16" s="2">
-        <v>0</v>
-      </c>
-      <c r="L16" s="2">
         <v>1</v>
       </c>
-      <c r="M16" s="5">
+      <c r="L16" s="5">
         <f t="shared" si="0"/>
         <v>7.6</v>
       </c>
-      <c r="N16" s="2" t="s">
-        <v>84</v>
-      </c>
-      <c r="O16" s="2" t="str">
+      <c r="M16" s="2" t="s">
+        <v>83</v>
+      </c>
+      <c r="N16" s="2" t="str">
         <f t="shared" si="1"/>
         <v>贡献 1 粒进球 / 送出 1 次助攻</v>
       </c>
     </row>
-    <row r="17" ht="23" customHeight="1" spans="1:15">
+    <row r="17" ht="23" customHeight="1" spans="1:14">
       <c r="A17" s="3">
         <v>16</v>
       </c>
       <c r="B17" s="3" t="s">
+        <v>84</v>
+      </c>
+      <c r="C17" s="3" t="s">
         <v>85</v>
-      </c>
-      <c r="C17" s="3" t="s">
-        <v>86</v>
       </c>
       <c r="D17" s="3">
         <v>66</v>
       </c>
       <c r="E17" s="3" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="F17" s="3" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="G17" s="3">
         <v>1</v>
@@ -2552,39 +2501,36 @@
       <c r="K17" s="3">
         <v>0</v>
       </c>
-      <c r="L17" s="3">
-        <v>0</v>
-      </c>
-      <c r="M17" s="6">
+      <c r="L17" s="6">
         <f t="shared" si="0"/>
         <v>6.1</v>
       </c>
-      <c r="N17" s="3" t="s">
-        <v>87</v>
-      </c>
-      <c r="O17" s="3" t="str">
+      <c r="M17" s="3" t="s">
+        <v>86</v>
+      </c>
+      <c r="N17" s="3" t="str">
         <f t="shared" si="1"/>
         <v>累计出场 1 场</v>
       </c>
     </row>
-    <row r="18" ht="23" customHeight="1" spans="1:15">
+    <row r="18" ht="23" customHeight="1" spans="1:14">
       <c r="A18" s="2">
         <v>17</v>
       </c>
       <c r="B18" s="2" t="s">
+        <v>87</v>
+      </c>
+      <c r="C18" s="2" t="s">
         <v>88</v>
-      </c>
-      <c r="C18" s="2" t="s">
-        <v>89</v>
       </c>
       <c r="D18" s="2">
         <v>15</v>
       </c>
       <c r="E18" s="2" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="F18" s="2" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="G18" s="2">
         <v>2</v>
@@ -2601,23 +2547,20 @@
       <c r="K18" s="2">
         <v>0</v>
       </c>
-      <c r="L18" s="2">
-        <v>0</v>
-      </c>
-      <c r="M18" s="5">
+      <c r="L18" s="5">
         <f t="shared" si="0"/>
         <v>6.2</v>
       </c>
-      <c r="N18" s="2" t="s">
-        <v>53</v>
-      </c>
-      <c r="O18" s="2" t="str">
+      <c r="M18" s="2" t="s">
+        <v>52</v>
+      </c>
+      <c r="N18" s="2" t="str">
         <f t="shared" si="1"/>
         <v>累计出场 2 场</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData" ref="A1:O18" etc:filterBottomFollowUsedRange="0">
+  <autoFilter xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData" ref="A1:N18" etc:filterBottomFollowUsedRange="0">
     <extLst/>
   </autoFilter>
   <conditionalFormatting sqref="M2:M18">
@@ -2652,82 +2595,82 @@
   <sheetData>
     <row r="1" ht="26" customHeight="1" spans="1:6">
       <c r="A1" s="1" t="s">
+        <v>90</v>
+      </c>
+      <c r="B1" s="1" t="s">
         <v>91</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="C1" s="1" t="s">
         <v>92</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="D1" s="1" t="s">
         <v>93</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="E1" s="1" t="s">
         <v>94</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="F1" s="1" t="s">
         <v>95</v>
       </c>
-      <c r="F1" s="1" t="s">
+    </row>
+    <row r="2" ht="27" customHeight="1" spans="1:6">
+      <c r="A2" s="2" t="s">
         <v>96</v>
       </c>
-    </row>
-    <row r="2" ht="27" spans="1:6">
-      <c r="A2" s="2" t="s">
+      <c r="B2" s="2" t="s">
         <v>97</v>
       </c>
-      <c r="B2" s="2" t="s">
+      <c r="C2" s="2" t="s">
         <v>98</v>
       </c>
-      <c r="C2" s="2" t="s">
+      <c r="D2" s="2" t="s">
+        <v>98</v>
+      </c>
+      <c r="E2" s="2" t="s">
         <v>99</v>
       </c>
-      <c r="D2" s="2" t="s">
-        <v>99</v>
-      </c>
-      <c r="E2" s="2" t="s">
+      <c r="F2" s="2" t="s">
         <v>100</v>
       </c>
-      <c r="F2" s="2" t="s">
+    </row>
+    <row r="3" ht="27" customHeight="1" spans="1:6">
+      <c r="A3" s="3" t="s">
         <v>101</v>
       </c>
-    </row>
-    <row r="3" ht="27" spans="1:6">
-      <c r="A3" s="3" t="s">
+      <c r="B3" s="3" t="s">
+        <v>97</v>
+      </c>
+      <c r="C3" s="3" t="s">
         <v>102</v>
       </c>
-      <c r="B3" s="3" t="s">
-        <v>98</v>
-      </c>
-      <c r="C3" s="3" t="s">
+      <c r="D3" s="3" t="s">
+        <v>102</v>
+      </c>
+      <c r="E3" s="3" t="s">
         <v>103</v>
       </c>
-      <c r="D3" s="3" t="s">
-        <v>103</v>
-      </c>
-      <c r="E3" s="3" t="s">
+      <c r="F3" s="3" t="s">
         <v>104</v>
-      </c>
-      <c r="F3" s="3" t="s">
-        <v>105</v>
       </c>
     </row>
     <row r="4" spans="1:6">
       <c r="A4" s="2" t="s">
+        <v>105</v>
+      </c>
+      <c r="B4" s="2" t="s">
         <v>106</v>
       </c>
-      <c r="B4" s="2" t="s">
+      <c r="C4" s="2" t="s">
         <v>107</v>
       </c>
-      <c r="C4" s="2" t="s">
+      <c r="D4" s="2" t="s">
+        <v>107</v>
+      </c>
+      <c r="E4" s="2" t="s">
         <v>108</v>
       </c>
-      <c r="D4" s="2" t="s">
-        <v>108</v>
-      </c>
-      <c r="E4" s="2" t="s">
+      <c r="F4" s="2" t="s">
         <v>109</v>
-      </c>
-      <c r="F4" s="2" t="s">
-        <v>110</v>
       </c>
     </row>
   </sheetData>
@@ -2758,350 +2701,350 @@
   <sheetData>
     <row r="1" ht="26" customHeight="1" spans="1:9">
       <c r="A1" s="1" t="s">
+        <v>110</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>92</v>
+      </c>
+      <c r="C1" s="1" t="s">
         <v>111</v>
       </c>
-      <c r="B1" s="1" t="s">
-        <v>93</v>
-      </c>
-      <c r="C1" s="1" t="s">
+      <c r="D1" s="1" t="s">
         <v>112</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="E1" s="1" t="s">
         <v>113</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="F1" s="1" t="s">
         <v>114</v>
       </c>
-      <c r="F1" s="1" t="s">
+      <c r="G1" s="1" t="s">
         <v>115</v>
       </c>
-      <c r="G1" s="1" t="s">
+      <c r="H1" s="1" t="s">
         <v>116</v>
       </c>
-      <c r="H1" s="1" t="s">
+      <c r="I1" s="1" t="s">
         <v>117</v>
-      </c>
-      <c r="I1" s="1" t="s">
-        <v>118</v>
       </c>
     </row>
     <row r="2" spans="1:9">
       <c r="A2" s="2" t="s">
+        <v>118</v>
+      </c>
+      <c r="B2" s="2" t="s">
+        <v>107</v>
+      </c>
+      <c r="C2" s="2" t="s">
         <v>119</v>
       </c>
-      <c r="B2" s="2" t="s">
-        <v>108</v>
-      </c>
-      <c r="C2" s="2" t="s">
+      <c r="D2" s="2" t="s">
         <v>120</v>
       </c>
-      <c r="D2" s="2" t="s">
+      <c r="E2" s="2" t="s">
         <v>121</v>
       </c>
-      <c r="E2" s="2" t="s">
+      <c r="F2" s="2" t="s">
         <v>122</v>
       </c>
-      <c r="F2" s="2" t="s">
+      <c r="G2" s="2" t="s">
         <v>123</v>
       </c>
-      <c r="G2" s="2" t="s">
+      <c r="H2" s="2" t="s">
         <v>124</v>
       </c>
-      <c r="H2" s="2" t="s">
+      <c r="I2" s="2" t="s">
         <v>125</v>
-      </c>
-      <c r="I2" s="2" t="s">
-        <v>126</v>
       </c>
     </row>
     <row r="3" spans="1:9">
       <c r="A3" s="3" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="B3" s="3" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="C3" s="3" t="s">
+        <v>126</v>
+      </c>
+      <c r="D3" s="3" t="s">
         <v>127</v>
       </c>
-      <c r="D3" s="3" t="s">
+      <c r="E3" s="3" t="s">
         <v>128</v>
       </c>
-      <c r="E3" s="3" t="s">
+      <c r="F3" s="3" t="s">
+        <v>122</v>
+      </c>
+      <c r="G3" s="3" t="s">
+        <v>123</v>
+      </c>
+      <c r="H3" s="3" t="s">
         <v>129</v>
       </c>
-      <c r="F3" s="3" t="s">
-        <v>123</v>
-      </c>
-      <c r="G3" s="3" t="s">
-        <v>124</v>
-      </c>
-      <c r="H3" s="3" t="s">
+      <c r="I3" s="3" t="s">
         <v>130</v>
-      </c>
-      <c r="I3" s="3" t="s">
-        <v>131</v>
       </c>
     </row>
     <row r="4" spans="1:9">
       <c r="A4" s="2" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="B4" s="2" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="C4" s="2" t="s">
+        <v>131</v>
+      </c>
+      <c r="D4" s="2" t="s">
         <v>132</v>
       </c>
-      <c r="D4" s="2" t="s">
+      <c r="E4" s="2" t="s">
         <v>133</v>
       </c>
-      <c r="E4" s="2" t="s">
+      <c r="F4" s="2" t="s">
+        <v>122</v>
+      </c>
+      <c r="G4" s="2" t="s">
+        <v>123</v>
+      </c>
+      <c r="H4" s="2" t="s">
         <v>134</v>
       </c>
-      <c r="F4" s="2" t="s">
+      <c r="I4" s="2" t="s">
+        <v>135</v>
+      </c>
+    </row>
+    <row r="5" ht="27" customHeight="1" spans="1:9">
+      <c r="A5" s="3" t="s">
+        <v>118</v>
+      </c>
+      <c r="B5" s="3" t="s">
+        <v>102</v>
+      </c>
+      <c r="C5" s="3" t="s">
+        <v>136</v>
+      </c>
+      <c r="D5" s="3" t="s">
+        <v>132</v>
+      </c>
+      <c r="E5" s="3" t="s">
+        <v>137</v>
+      </c>
+      <c r="F5" s="3" t="s">
+        <v>138</v>
+      </c>
+      <c r="G5" s="3" t="s">
         <v>123</v>
       </c>
-      <c r="G4" s="2" t="s">
-        <v>124</v>
-      </c>
-      <c r="H4" s="2" t="s">
-        <v>135</v>
-      </c>
-      <c r="I4" s="2" t="s">
-        <v>136</v>
-      </c>
-    </row>
-    <row r="5" ht="27" spans="1:9">
-      <c r="A5" s="3" t="s">
-        <v>119</v>
-      </c>
-      <c r="B5" s="3" t="s">
-        <v>103</v>
-      </c>
-      <c r="C5" s="3" t="s">
-        <v>137</v>
-      </c>
-      <c r="D5" s="3" t="s">
-        <v>133</v>
-      </c>
-      <c r="E5" s="3" t="s">
-        <v>138</v>
-      </c>
-      <c r="F5" s="3" t="s">
+      <c r="H5" s="3" t="s">
         <v>139</v>
       </c>
-      <c r="G5" s="3" t="s">
-        <v>124</v>
-      </c>
-      <c r="H5" s="3" t="s">
+      <c r="I5" s="3" t="s">
         <v>140</v>
-      </c>
-      <c r="I5" s="3" t="s">
-        <v>141</v>
       </c>
     </row>
     <row r="6" spans="1:9">
       <c r="A6" s="2" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="B6" s="2" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="C6" s="2" t="s">
+        <v>141</v>
+      </c>
+      <c r="D6" s="2" t="s">
         <v>142</v>
       </c>
-      <c r="D6" s="2" t="s">
+      <c r="E6" s="2" t="s">
         <v>143</v>
       </c>
-      <c r="E6" s="2" t="s">
+      <c r="F6" s="2" t="s">
+        <v>122</v>
+      </c>
+      <c r="G6" s="2" t="s">
+        <v>123</v>
+      </c>
+      <c r="H6" s="2" t="s">
+        <v>124</v>
+      </c>
+      <c r="I6" s="2" t="s">
         <v>144</v>
-      </c>
-      <c r="F6" s="2" t="s">
-        <v>123</v>
-      </c>
-      <c r="G6" s="2" t="s">
-        <v>124</v>
-      </c>
-      <c r="H6" s="2" t="s">
-        <v>125</v>
-      </c>
-      <c r="I6" s="2" t="s">
-        <v>145</v>
       </c>
     </row>
     <row r="7" spans="1:9">
       <c r="A7" s="3" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="B7" s="3" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="C7" s="3" t="s">
+        <v>145</v>
+      </c>
+      <c r="D7" s="3" t="s">
         <v>146</v>
       </c>
-      <c r="D7" s="3" t="s">
+      <c r="E7" s="3" t="s">
         <v>147</v>
       </c>
-      <c r="E7" s="3" t="s">
+      <c r="F7" s="3" t="s">
+        <v>122</v>
+      </c>
+      <c r="G7" s="3" t="s">
+        <v>123</v>
+      </c>
+      <c r="H7" s="3" t="s">
         <v>148</v>
       </c>
-      <c r="F7" s="3" t="s">
-        <v>123</v>
-      </c>
-      <c r="G7" s="3" t="s">
-        <v>124</v>
-      </c>
-      <c r="H7" s="3" t="s">
+      <c r="I7" s="3" t="s">
         <v>149</v>
-      </c>
-      <c r="I7" s="3" t="s">
-        <v>150</v>
       </c>
     </row>
     <row r="8" spans="1:9">
       <c r="A8" s="2" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="B8" s="2" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="C8" s="2" t="s">
+        <v>150</v>
+      </c>
+      <c r="D8" s="2" t="s">
         <v>151</v>
       </c>
-      <c r="D8" s="2" t="s">
+      <c r="E8" s="2" t="s">
         <v>152</v>
       </c>
-      <c r="E8" s="2" t="s">
+      <c r="F8" s="2" t="s">
+        <v>138</v>
+      </c>
+      <c r="G8" s="2" t="s">
+        <v>123</v>
+      </c>
+      <c r="H8" s="2" t="s">
         <v>153</v>
       </c>
-      <c r="F8" s="2" t="s">
-        <v>139</v>
-      </c>
-      <c r="G8" s="2" t="s">
-        <v>124</v>
-      </c>
-      <c r="H8" s="2" t="s">
+      <c r="I8" s="2" t="s">
         <v>154</v>
-      </c>
-      <c r="I8" s="2" t="s">
-        <v>155</v>
       </c>
     </row>
     <row r="9" spans="1:9">
       <c r="A9" s="3" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="B9" s="3" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="C9" s="3" t="s">
+        <v>155</v>
+      </c>
+      <c r="D9" s="3" t="s">
         <v>156</v>
       </c>
-      <c r="D9" s="3" t="s">
+      <c r="E9" s="3" t="s">
+        <v>137</v>
+      </c>
+      <c r="F9" s="3" t="s">
+        <v>138</v>
+      </c>
+      <c r="G9" s="3" t="s">
+        <v>123</v>
+      </c>
+      <c r="H9" s="3" t="s">
         <v>157</v>
       </c>
-      <c r="E9" s="3" t="s">
-        <v>138</v>
-      </c>
-      <c r="F9" s="3" t="s">
-        <v>139</v>
-      </c>
-      <c r="G9" s="3" t="s">
-        <v>124</v>
-      </c>
-      <c r="H9" s="3" t="s">
+      <c r="I9" s="3" t="s">
         <v>158</v>
-      </c>
-      <c r="I9" s="3" t="s">
-        <v>159</v>
       </c>
     </row>
     <row r="10" spans="1:9">
       <c r="A10" s="2" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="B10" s="2" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="C10" s="2" t="s">
+        <v>159</v>
+      </c>
+      <c r="D10" s="2" t="s">
         <v>160</v>
       </c>
-      <c r="D10" s="2" t="s">
+      <c r="E10" s="2" t="s">
         <v>161</v>
       </c>
-      <c r="E10" s="2" t="s">
+      <c r="F10" s="2" t="s">
+        <v>122</v>
+      </c>
+      <c r="G10" s="2" t="s">
+        <v>123</v>
+      </c>
+      <c r="H10" s="2" t="s">
+        <v>124</v>
+      </c>
+      <c r="I10" s="2" t="s">
         <v>162</v>
-      </c>
-      <c r="F10" s="2" t="s">
-        <v>123</v>
-      </c>
-      <c r="G10" s="2" t="s">
-        <v>124</v>
-      </c>
-      <c r="H10" s="2" t="s">
-        <v>125</v>
-      </c>
-      <c r="I10" s="2" t="s">
-        <v>163</v>
       </c>
     </row>
     <row r="11" spans="1:9">
       <c r="A11" s="3" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="B11" s="3" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="C11" s="3" t="s">
+        <v>163</v>
+      </c>
+      <c r="D11" s="3" t="s">
+        <v>120</v>
+      </c>
+      <c r="E11" s="3" t="s">
         <v>164</v>
       </c>
-      <c r="D11" s="3" t="s">
-        <v>121</v>
-      </c>
-      <c r="E11" s="3" t="s">
+      <c r="F11" s="3" t="s">
+        <v>122</v>
+      </c>
+      <c r="G11" s="3" t="s">
+        <v>123</v>
+      </c>
+      <c r="H11" s="3" t="s">
         <v>165</v>
       </c>
-      <c r="F11" s="3" t="s">
+      <c r="I11" s="3" t="s">
+        <v>166</v>
+      </c>
+    </row>
+    <row r="12" ht="27" customHeight="1" spans="1:9">
+      <c r="A12" s="2" t="s">
+        <v>118</v>
+      </c>
+      <c r="B12" s="2" t="s">
+        <v>98</v>
+      </c>
+      <c r="C12" s="2" t="s">
+        <v>167</v>
+      </c>
+      <c r="D12" s="2" t="s">
+        <v>132</v>
+      </c>
+      <c r="E12" s="2" t="s">
+        <v>168</v>
+      </c>
+      <c r="F12" s="2" t="s">
+        <v>122</v>
+      </c>
+      <c r="G12" s="2" t="s">
         <v>123</v>
       </c>
-      <c r="G11" s="3" t="s">
-        <v>124</v>
-      </c>
-      <c r="H11" s="3" t="s">
-        <v>166</v>
-      </c>
-      <c r="I11" s="3" t="s">
-        <v>167</v>
-      </c>
-    </row>
-    <row r="12" ht="27" spans="1:9">
-      <c r="A12" s="2" t="s">
-        <v>119</v>
-      </c>
-      <c r="B12" s="2" t="s">
-        <v>99</v>
-      </c>
-      <c r="C12" s="2" t="s">
-        <v>168</v>
-      </c>
-      <c r="D12" s="2" t="s">
-        <v>133</v>
-      </c>
-      <c r="E12" s="2" t="s">
+      <c r="H12" s="2" t="s">
         <v>169</v>
       </c>
-      <c r="F12" s="2" t="s">
-        <v>123</v>
-      </c>
-      <c r="G12" s="2" t="s">
-        <v>124</v>
-      </c>
-      <c r="H12" s="2" t="s">
+      <c r="I12" s="2" t="s">
         <v>170</v>
-      </c>
-      <c r="I12" s="2" t="s">
-        <v>171</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Reward defensive contribution in ratings
</commit_message>
<xml_diff>
--- a/data/生康足球队数据源.xlsx
+++ b/data/生康足球队数据源.xlsx
@@ -13,7 +13,7 @@
     <sheet name="赛程" sheetId="4" r:id="rId4"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">球员数据!$A$1:$N$18</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">球员数据!$A$1:$O$18</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">赛事索引!$A$1:$F$4</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">赛程!$A$1:$I$12</definedName>
   </definedNames>
@@ -35,7 +35,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="244" uniqueCount="171">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="245" uniqueCount="172">
   <si>
     <t>生康足球队 · 球员数据汇总</t>
   </si>
@@ -107,6 +107,9 @@
   </si>
   <si>
     <t>零封</t>
+  </si>
+  <si>
+    <t>低失球场</t>
   </si>
   <si>
     <t>评分</t>
@@ -1718,7 +1721,7 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
-  <dimension ref="A1:N18"/>
+  <dimension ref="A1:O18"/>
   <sheetFormatPr defaultColWidth="9" defaultRowHeight="13.5"/>
   <cols>
     <col min="1" max="1" width="8" customWidth="1"/>
@@ -1728,12 +1731,13 @@
     <col min="5" max="5" width="10" customWidth="1"/>
     <col min="6" max="6" width="17" customWidth="1"/>
     <col min="7" max="11" width="9" customWidth="1"/>
-    <col min="12" max="12" width="12" customWidth="1"/>
-    <col min="13" max="13" width="20" customWidth="1"/>
-    <col min="14" max="15" width="28" customWidth="1"/>
+    <col min="12" max="12" width="11" customWidth="1"/>
+    <col min="13" max="13" width="12" customWidth="1"/>
+    <col min="14" max="14" width="20" customWidth="1"/>
+    <col min="15" max="15" width="28" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" ht="26" customHeight="1" spans="1:14">
+    <row r="1" ht="26" customHeight="1" spans="1:15">
       <c r="A1" s="4" t="s">
         <v>13</v>
       </c>
@@ -1767,7 +1771,7 @@
       <c r="K1" s="4" t="s">
         <v>23</v>
       </c>
-      <c r="L1" s="4" t="s">
+      <c r="L1" s="1" t="s">
         <v>24</v>
       </c>
       <c r="M1" s="4" t="s">
@@ -1776,25 +1780,28 @@
       <c r="N1" s="4" t="s">
         <v>26</v>
       </c>
-    </row>
-    <row r="2" ht="23" customHeight="1" spans="1:14">
+      <c r="O1" s="4" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="2" ht="23" customHeight="1" spans="1:15">
       <c r="A2" s="2">
         <v>1</v>
       </c>
       <c r="B2" s="2" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="C2" s="2" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="D2" s="2">
         <v>6</v>
       </c>
       <c r="E2" s="2" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="F2" s="2" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="G2" s="2">
         <v>11</v>
@@ -1811,36 +1818,39 @@
       <c r="K2" s="2">
         <v>0</v>
       </c>
-      <c r="L2" s="5">
-        <f t="shared" ref="L2:L18" si="0">ROUND(MIN(9.5,MAX(6,6+G2*0.08+H2*0.35+I2*0.25+J2*0.25+K2*0.15)),1)</f>
-        <v>7.1</v>
-      </c>
-      <c r="M2" s="2" t="s">
-        <v>31</v>
-      </c>
-      <c r="N2" s="2" t="str">
-        <f t="shared" ref="N2:N18" si="1">IF(H2&gt;0,IF(I2&gt;0,"贡献 "&amp;H2&amp;" 粒进球 / 送出 "&amp;I2&amp;" 次助攻","贡献 "&amp;H2&amp;" 粒进球"),IF(I2&gt;0,"送出 "&amp;I2&amp;" 次助攻","累计出场 "&amp;G2&amp;" 场"))</f>
+      <c r="L2" s="2">
+        <v>0</v>
+      </c>
+      <c r="M2" s="5">
+        <f t="shared" ref="M2:M18" si="0">ROUND(MIN(9.5,MAX(6,6+G2*0.08+H2*0.35+I2*0.25+J2*0.25+K2*0.15+IF(E2="DF",G2*0.06+K2*0.35+L2*0.15,0))),1)</f>
+        <v>7.8</v>
+      </c>
+      <c r="N2" s="2" t="s">
+        <v>32</v>
+      </c>
+      <c r="O2" s="2" t="str">
+        <f t="shared" ref="O2:O18" si="1">IF(H2&gt;0,IF(I2&gt;0,"贡献 "&amp;H2&amp;" 粒进球 / 送出 "&amp;I2&amp;" 次助攻","贡献 "&amp;H2&amp;" 粒进球"),IF(I2&gt;0,"送出 "&amp;I2&amp;" 次助攻","累计出场 "&amp;G2&amp;" 场"))</f>
         <v>送出 1 次助攻</v>
       </c>
     </row>
-    <row r="3" ht="23" customHeight="1" spans="1:14">
+    <row r="3" ht="23" customHeight="1" spans="1:15">
       <c r="A3" s="3">
         <v>2</v>
       </c>
       <c r="B3" s="3" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="C3" s="3" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="D3" s="3">
         <v>10</v>
       </c>
       <c r="E3" s="3" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="F3" s="3" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="G3" s="3">
         <v>4</v>
@@ -1857,710 +1867,758 @@
       <c r="K3" s="3">
         <v>0</v>
       </c>
-      <c r="L3" s="6">
+      <c r="L3" s="3">
+        <v>0</v>
+      </c>
+      <c r="M3" s="6">
+        <f t="shared" si="0"/>
+        <v>6.6</v>
+      </c>
+      <c r="N3" s="3" t="s">
+        <v>36</v>
+      </c>
+      <c r="O3" s="3" t="str">
+        <f t="shared" si="1"/>
+        <v>累计出场 4 场</v>
+      </c>
+    </row>
+    <row r="4" ht="23" customHeight="1" spans="1:15">
+      <c r="A4" s="2">
+        <v>3</v>
+      </c>
+      <c r="B4" s="2" t="s">
+        <v>37</v>
+      </c>
+      <c r="C4" s="2" t="s">
+        <v>38</v>
+      </c>
+      <c r="D4" s="2">
+        <v>29</v>
+      </c>
+      <c r="E4" s="2" t="s">
+        <v>30</v>
+      </c>
+      <c r="F4" s="2" t="s">
+        <v>39</v>
+      </c>
+      <c r="G4" s="2">
+        <v>9</v>
+      </c>
+      <c r="H4" s="2">
+        <v>0</v>
+      </c>
+      <c r="I4" s="2">
+        <v>0</v>
+      </c>
+      <c r="J4" s="2">
+        <v>0</v>
+      </c>
+      <c r="K4" s="2">
+        <v>0</v>
+      </c>
+      <c r="L4" s="2">
+        <v>0</v>
+      </c>
+      <c r="M4" s="5">
+        <f t="shared" si="0"/>
+        <v>7.3</v>
+      </c>
+      <c r="N4" s="2" t="s">
+        <v>40</v>
+      </c>
+      <c r="O4" s="2" t="str">
+        <f t="shared" si="1"/>
+        <v>累计出场 9 场</v>
+      </c>
+    </row>
+    <row r="5" ht="23" customHeight="1" spans="1:15">
+      <c r="A5" s="3">
+        <v>4</v>
+      </c>
+      <c r="B5" s="3" t="s">
+        <v>41</v>
+      </c>
+      <c r="C5" s="3" t="s">
+        <v>42</v>
+      </c>
+      <c r="D5" s="3">
+        <v>0</v>
+      </c>
+      <c r="E5" s="3" t="s">
+        <v>43</v>
+      </c>
+      <c r="F5" s="3" t="s">
+        <v>43</v>
+      </c>
+      <c r="G5" s="3">
+        <v>8</v>
+      </c>
+      <c r="H5" s="3">
+        <v>0</v>
+      </c>
+      <c r="I5" s="3">
+        <v>0</v>
+      </c>
+      <c r="J5" s="3">
+        <v>0</v>
+      </c>
+      <c r="K5" s="3">
+        <v>1</v>
+      </c>
+      <c r="L5" s="3">
+        <v>0</v>
+      </c>
+      <c r="M5" s="6">
+        <f t="shared" si="0"/>
+        <v>6.8</v>
+      </c>
+      <c r="N5" s="3" t="s">
+        <v>44</v>
+      </c>
+      <c r="O5" s="3" t="str">
+        <f t="shared" si="1"/>
+        <v>累计出场 8 场</v>
+      </c>
+    </row>
+    <row r="6" ht="23" customHeight="1" spans="1:15">
+      <c r="A6" s="2">
+        <v>5</v>
+      </c>
+      <c r="B6" s="2" t="s">
+        <v>45</v>
+      </c>
+      <c r="C6" s="2" t="s">
+        <v>46</v>
+      </c>
+      <c r="D6" s="2">
+        <v>23</v>
+      </c>
+      <c r="E6" s="2" t="s">
+        <v>47</v>
+      </c>
+      <c r="F6" s="2" t="s">
+        <v>48</v>
+      </c>
+      <c r="G6" s="2">
+        <v>8</v>
+      </c>
+      <c r="H6" s="2">
+        <v>0</v>
+      </c>
+      <c r="I6" s="2">
+        <v>0</v>
+      </c>
+      <c r="J6" s="2">
+        <v>0</v>
+      </c>
+      <c r="K6" s="2">
+        <v>0</v>
+      </c>
+      <c r="L6" s="2">
+        <v>0</v>
+      </c>
+      <c r="M6" s="5">
+        <f t="shared" si="0"/>
+        <v>6.6</v>
+      </c>
+      <c r="N6" s="2" t="s">
+        <v>49</v>
+      </c>
+      <c r="O6" s="2" t="str">
+        <f t="shared" si="1"/>
+        <v>累计出场 8 场</v>
+      </c>
+    </row>
+    <row r="7" ht="23" customHeight="1" spans="1:15">
+      <c r="A7" s="3">
+        <v>6</v>
+      </c>
+      <c r="B7" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="C7" s="3" t="s">
+        <v>51</v>
+      </c>
+      <c r="D7" s="3">
+        <v>9</v>
+      </c>
+      <c r="E7" s="3" t="s">
+        <v>30</v>
+      </c>
+      <c r="F7" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="G7" s="3">
+        <v>0</v>
+      </c>
+      <c r="H7" s="3">
+        <v>0</v>
+      </c>
+      <c r="I7" s="3">
+        <v>0</v>
+      </c>
+      <c r="J7" s="3">
+        <v>0</v>
+      </c>
+      <c r="K7" s="3">
+        <v>0</v>
+      </c>
+      <c r="L7" s="3">
+        <v>0</v>
+      </c>
+      <c r="M7" s="6">
+        <f t="shared" si="0"/>
+        <v>6</v>
+      </c>
+      <c r="N7" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="O7" s="3" t="str">
+        <f t="shared" si="1"/>
+        <v>累计出场 0 场</v>
+      </c>
+    </row>
+    <row r="8" ht="23" customHeight="1" spans="1:15">
+      <c r="A8" s="2">
+        <v>7</v>
+      </c>
+      <c r="B8" s="2" t="s">
+        <v>54</v>
+      </c>
+      <c r="C8" s="2" t="s">
+        <v>55</v>
+      </c>
+      <c r="D8" s="2">
+        <v>15</v>
+      </c>
+      <c r="E8" s="2" t="s">
+        <v>47</v>
+      </c>
+      <c r="F8" s="2" t="s">
+        <v>56</v>
+      </c>
+      <c r="G8" s="2">
+        <v>11</v>
+      </c>
+      <c r="H8" s="2">
+        <v>6</v>
+      </c>
+      <c r="I8" s="2">
+        <v>1</v>
+      </c>
+      <c r="J8" s="2">
+        <v>0</v>
+      </c>
+      <c r="K8" s="2">
+        <v>0</v>
+      </c>
+      <c r="L8" s="2">
+        <v>0</v>
+      </c>
+      <c r="M8" s="5">
+        <f t="shared" si="0"/>
+        <v>9.2</v>
+      </c>
+      <c r="N8" s="2" t="s">
+        <v>57</v>
+      </c>
+      <c r="O8" s="2" t="str">
+        <f t="shared" si="1"/>
+        <v>贡献 6 粒进球 / 送出 1 次助攻</v>
+      </c>
+    </row>
+    <row r="9" ht="23" customHeight="1" spans="1:15">
+      <c r="A9" s="3">
+        <v>8</v>
+      </c>
+      <c r="B9" s="3" t="s">
+        <v>58</v>
+      </c>
+      <c r="C9" s="3" t="s">
+        <v>59</v>
+      </c>
+      <c r="D9" s="3">
+        <v>8</v>
+      </c>
+      <c r="E9" s="3" t="s">
+        <v>60</v>
+      </c>
+      <c r="F9" s="3" t="s">
+        <v>61</v>
+      </c>
+      <c r="G9" s="3">
+        <v>8</v>
+      </c>
+      <c r="H9" s="3">
+        <v>2</v>
+      </c>
+      <c r="I9" s="3">
+        <v>3</v>
+      </c>
+      <c r="J9" s="3">
+        <v>0</v>
+      </c>
+      <c r="K9" s="3">
+        <v>0</v>
+      </c>
+      <c r="L9" s="3">
+        <v>0</v>
+      </c>
+      <c r="M9" s="6">
+        <f t="shared" si="0"/>
+        <v>8.1</v>
+      </c>
+      <c r="N9" s="3" t="s">
+        <v>62</v>
+      </c>
+      <c r="O9" s="3" t="str">
+        <f t="shared" si="1"/>
+        <v>贡献 2 粒进球 / 送出 3 次助攻</v>
+      </c>
+    </row>
+    <row r="10" ht="23" customHeight="1" spans="1:15">
+      <c r="A10" s="2">
+        <v>9</v>
+      </c>
+      <c r="B10" s="2" t="s">
+        <v>63</v>
+      </c>
+      <c r="C10" s="2" t="s">
+        <v>64</v>
+      </c>
+      <c r="D10" s="2">
+        <v>5</v>
+      </c>
+      <c r="E10" s="2" t="s">
+        <v>47</v>
+      </c>
+      <c r="F10" s="2" t="s">
+        <v>65</v>
+      </c>
+      <c r="G10" s="2">
+        <v>10</v>
+      </c>
+      <c r="H10" s="2">
+        <v>4</v>
+      </c>
+      <c r="I10" s="2">
+        <v>3</v>
+      </c>
+      <c r="J10" s="2">
+        <v>0</v>
+      </c>
+      <c r="K10" s="2">
+        <v>0</v>
+      </c>
+      <c r="L10" s="2">
+        <v>0</v>
+      </c>
+      <c r="M10" s="5">
+        <f t="shared" si="0"/>
+        <v>9</v>
+      </c>
+      <c r="N10" s="2" t="s">
+        <v>66</v>
+      </c>
+      <c r="O10" s="2" t="str">
+        <f t="shared" si="1"/>
+        <v>贡献 4 粒进球 / 送出 3 次助攻</v>
+      </c>
+    </row>
+    <row r="11" ht="23" customHeight="1" spans="1:15">
+      <c r="A11" s="3">
+        <v>10</v>
+      </c>
+      <c r="B11" s="3" t="s">
+        <v>67</v>
+      </c>
+      <c r="C11" s="3" t="s">
+        <v>68</v>
+      </c>
+      <c r="D11" s="3">
+        <v>17</v>
+      </c>
+      <c r="E11" s="3" t="s">
+        <v>30</v>
+      </c>
+      <c r="F11" s="3" t="s">
+        <v>31</v>
+      </c>
+      <c r="G11" s="3">
+        <v>6</v>
+      </c>
+      <c r="H11" s="3">
+        <v>0</v>
+      </c>
+      <c r="I11" s="3">
+        <v>0</v>
+      </c>
+      <c r="J11" s="3">
+        <v>0</v>
+      </c>
+      <c r="K11" s="3">
+        <v>0</v>
+      </c>
+      <c r="L11" s="3">
+        <v>0</v>
+      </c>
+      <c r="M11" s="6">
+        <f t="shared" si="0"/>
+        <v>6.8</v>
+      </c>
+      <c r="N11" s="3" t="s">
+        <v>69</v>
+      </c>
+      <c r="O11" s="3" t="str">
+        <f t="shared" si="1"/>
+        <v>累计出场 6 场</v>
+      </c>
+    </row>
+    <row r="12" ht="23" customHeight="1" spans="1:15">
+      <c r="A12" s="2">
+        <v>11</v>
+      </c>
+      <c r="B12" s="2" t="s">
+        <v>70</v>
+      </c>
+      <c r="C12" s="2" t="s">
+        <v>42</v>
+      </c>
+      <c r="D12" s="2">
+        <v>18</v>
+      </c>
+      <c r="E12" s="2" t="s">
+        <v>43</v>
+      </c>
+      <c r="F12" s="2" t="s">
+        <v>71</v>
+      </c>
+      <c r="G12" s="2">
+        <v>5</v>
+      </c>
+      <c r="H12" s="2">
+        <v>0</v>
+      </c>
+      <c r="I12" s="2">
+        <v>0</v>
+      </c>
+      <c r="J12" s="2">
+        <v>0</v>
+      </c>
+      <c r="K12" s="2">
+        <v>1</v>
+      </c>
+      <c r="L12" s="2">
+        <v>0</v>
+      </c>
+      <c r="M12" s="5">
+        <f t="shared" si="0"/>
+        <v>6.6</v>
+      </c>
+      <c r="N12" s="2" t="s">
+        <v>44</v>
+      </c>
+      <c r="O12" s="2" t="str">
+        <f t="shared" si="1"/>
+        <v>累计出场 5 场</v>
+      </c>
+    </row>
+    <row r="13" ht="23" customHeight="1" spans="1:15">
+      <c r="A13" s="3">
+        <v>12</v>
+      </c>
+      <c r="B13" s="3" t="s">
+        <v>72</v>
+      </c>
+      <c r="C13" s="3" t="s">
+        <v>73</v>
+      </c>
+      <c r="D13" s="3">
+        <v>19</v>
+      </c>
+      <c r="E13" s="3" t="s">
+        <v>30</v>
+      </c>
+      <c r="F13" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="G13" s="3">
+        <v>8</v>
+      </c>
+      <c r="H13" s="3">
+        <v>0</v>
+      </c>
+      <c r="I13" s="3">
+        <v>0</v>
+      </c>
+      <c r="J13" s="3">
+        <v>0</v>
+      </c>
+      <c r="K13" s="3">
+        <v>0</v>
+      </c>
+      <c r="L13" s="3">
+        <v>0</v>
+      </c>
+      <c r="M13" s="6">
+        <f t="shared" si="0"/>
+        <v>7.1</v>
+      </c>
+      <c r="N13" s="3" t="s">
+        <v>74</v>
+      </c>
+      <c r="O13" s="3" t="str">
+        <f t="shared" si="1"/>
+        <v>累计出场 8 场</v>
+      </c>
+    </row>
+    <row r="14" ht="23" customHeight="1" spans="1:15">
+      <c r="A14" s="2">
+        <v>13</v>
+      </c>
+      <c r="B14" s="2" t="s">
+        <v>75</v>
+      </c>
+      <c r="C14" s="2" t="s">
+        <v>76</v>
+      </c>
+      <c r="D14" s="2">
+        <v>25</v>
+      </c>
+      <c r="E14" s="2" t="s">
+        <v>60</v>
+      </c>
+      <c r="F14" s="2" t="s">
+        <v>77</v>
+      </c>
+      <c r="G14" s="2">
+        <v>6</v>
+      </c>
+      <c r="H14" s="2">
+        <v>0</v>
+      </c>
+      <c r="I14" s="2">
+        <v>0</v>
+      </c>
+      <c r="J14" s="2">
+        <v>0</v>
+      </c>
+      <c r="K14" s="2">
+        <v>0</v>
+      </c>
+      <c r="L14" s="2">
+        <v>0</v>
+      </c>
+      <c r="M14" s="5">
+        <f t="shared" si="0"/>
+        <v>6.5</v>
+      </c>
+      <c r="N14" s="2" t="s">
+        <v>69</v>
+      </c>
+      <c r="O14" s="2" t="str">
+        <f t="shared" si="1"/>
+        <v>累计出场 6 场</v>
+      </c>
+    </row>
+    <row r="15" ht="23" customHeight="1" spans="1:15">
+      <c r="A15" s="3">
+        <v>14</v>
+      </c>
+      <c r="B15" s="3" t="s">
+        <v>78</v>
+      </c>
+      <c r="C15" s="3" t="s">
+        <v>79</v>
+      </c>
+      <c r="D15" s="3">
+        <v>66</v>
+      </c>
+      <c r="E15" s="3" t="s">
+        <v>30</v>
+      </c>
+      <c r="F15" s="3" t="s">
+        <v>80</v>
+      </c>
+      <c r="G15" s="3">
+        <v>3</v>
+      </c>
+      <c r="H15" s="3">
+        <v>0</v>
+      </c>
+      <c r="I15" s="3">
+        <v>0</v>
+      </c>
+      <c r="J15" s="3">
+        <v>0</v>
+      </c>
+      <c r="K15" s="3">
+        <v>0</v>
+      </c>
+      <c r="L15" s="3">
+        <v>0</v>
+      </c>
+      <c r="M15" s="6">
+        <f t="shared" si="0"/>
+        <v>6.4</v>
+      </c>
+      <c r="N15" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="O15" s="3" t="str">
+        <f t="shared" si="1"/>
+        <v>累计出场 3 场</v>
+      </c>
+    </row>
+    <row r="16" ht="23" customHeight="1" spans="1:15">
+      <c r="A16" s="2">
+        <v>15</v>
+      </c>
+      <c r="B16" s="2" t="s">
+        <v>81</v>
+      </c>
+      <c r="C16" s="2" t="s">
+        <v>82</v>
+      </c>
+      <c r="D16" s="2">
+        <v>12</v>
+      </c>
+      <c r="E16" s="2" t="s">
+        <v>60</v>
+      </c>
+      <c r="F16" s="2" t="s">
+        <v>83</v>
+      </c>
+      <c r="G16" s="2">
+        <v>10</v>
+      </c>
+      <c r="H16" s="2">
+        <v>1</v>
+      </c>
+      <c r="I16" s="2">
+        <v>1</v>
+      </c>
+      <c r="J16" s="2">
+        <v>0</v>
+      </c>
+      <c r="K16" s="2">
+        <v>1</v>
+      </c>
+      <c r="L16" s="2">
+        <v>0</v>
+      </c>
+      <c r="M16" s="5">
+        <f t="shared" si="0"/>
+        <v>7.6</v>
+      </c>
+      <c r="N16" s="2" t="s">
+        <v>84</v>
+      </c>
+      <c r="O16" s="2" t="str">
+        <f t="shared" si="1"/>
+        <v>贡献 1 粒进球 / 送出 1 次助攻</v>
+      </c>
+    </row>
+    <row r="17" ht="23" customHeight="1" spans="1:15">
+      <c r="A17" s="3">
+        <v>16</v>
+      </c>
+      <c r="B17" s="3" t="s">
+        <v>85</v>
+      </c>
+      <c r="C17" s="3" t="s">
+        <v>86</v>
+      </c>
+      <c r="D17" s="3">
+        <v>66</v>
+      </c>
+      <c r="E17" s="3" t="s">
+        <v>43</v>
+      </c>
+      <c r="F17" s="3" t="s">
+        <v>43</v>
+      </c>
+      <c r="G17" s="3">
+        <v>1</v>
+      </c>
+      <c r="H17" s="3">
+        <v>0</v>
+      </c>
+      <c r="I17" s="3">
+        <v>0</v>
+      </c>
+      <c r="J17" s="3">
+        <v>0</v>
+      </c>
+      <c r="K17" s="3">
+        <v>0</v>
+      </c>
+      <c r="L17" s="3">
+        <v>0</v>
+      </c>
+      <c r="M17" s="6">
+        <f t="shared" si="0"/>
+        <v>6.1</v>
+      </c>
+      <c r="N17" s="3" t="s">
+        <v>87</v>
+      </c>
+      <c r="O17" s="3" t="str">
+        <f t="shared" si="1"/>
+        <v>累计出场 1 场</v>
+      </c>
+    </row>
+    <row r="18" ht="23" customHeight="1" spans="1:15">
+      <c r="A18" s="2">
+        <v>17</v>
+      </c>
+      <c r="B18" s="2" t="s">
+        <v>88</v>
+      </c>
+      <c r="C18" s="2" t="s">
+        <v>89</v>
+      </c>
+      <c r="D18" s="2">
+        <v>15</v>
+      </c>
+      <c r="E18" s="2" t="s">
+        <v>30</v>
+      </c>
+      <c r="F18" s="2" t="s">
+        <v>90</v>
+      </c>
+      <c r="G18" s="2">
+        <v>2</v>
+      </c>
+      <c r="H18" s="2">
+        <v>0</v>
+      </c>
+      <c r="I18" s="2">
+        <v>0</v>
+      </c>
+      <c r="J18" s="2">
+        <v>0</v>
+      </c>
+      <c r="K18" s="2">
+        <v>0</v>
+      </c>
+      <c r="L18" s="2">
+        <v>0</v>
+      </c>
+      <c r="M18" s="5">
         <f t="shared" si="0"/>
         <v>6.3</v>
       </c>
-      <c r="M3" s="3" t="s">
-        <v>35</v>
-      </c>
-      <c r="N3" s="3" t="str">
-        <f t="shared" si="1"/>
-        <v>累计出场 4 场</v>
-      </c>
-    </row>
-    <row r="4" ht="23" customHeight="1" spans="1:14">
-      <c r="A4" s="2">
-        <v>3</v>
-      </c>
-      <c r="B4" s="2" t="s">
-        <v>36</v>
-      </c>
-      <c r="C4" s="2" t="s">
-        <v>37</v>
-      </c>
-      <c r="D4" s="2">
-        <v>29</v>
-      </c>
-      <c r="E4" s="2" t="s">
-        <v>29</v>
-      </c>
-      <c r="F4" s="2" t="s">
-        <v>38</v>
-      </c>
-      <c r="G4" s="2">
-        <v>9</v>
-      </c>
-      <c r="H4" s="2">
-        <v>0</v>
-      </c>
-      <c r="I4" s="2">
-        <v>0</v>
-      </c>
-      <c r="J4" s="2">
-        <v>0</v>
-      </c>
-      <c r="K4" s="2">
-        <v>0</v>
-      </c>
-      <c r="L4" s="5">
-        <f t="shared" si="0"/>
-        <v>6.7</v>
-      </c>
-      <c r="M4" s="2" t="s">
-        <v>39</v>
-      </c>
-      <c r="N4" s="2" t="str">
-        <f t="shared" si="1"/>
-        <v>累计出场 9 场</v>
-      </c>
-    </row>
-    <row r="5" ht="23" customHeight="1" spans="1:14">
-      <c r="A5" s="3">
-        <v>4</v>
-      </c>
-      <c r="B5" s="3" t="s">
-        <v>40</v>
-      </c>
-      <c r="C5" s="3" t="s">
-        <v>41</v>
-      </c>
-      <c r="D5" s="3">
-        <v>0</v>
-      </c>
-      <c r="E5" s="3" t="s">
-        <v>42</v>
-      </c>
-      <c r="F5" s="3" t="s">
-        <v>42</v>
-      </c>
-      <c r="G5" s="3">
-        <v>8</v>
-      </c>
-      <c r="H5" s="3">
-        <v>0</v>
-      </c>
-      <c r="I5" s="3">
-        <v>0</v>
-      </c>
-      <c r="J5" s="3">
-        <v>0</v>
-      </c>
-      <c r="K5" s="3">
-        <v>1</v>
-      </c>
-      <c r="L5" s="6">
-        <f t="shared" si="0"/>
-        <v>6.8</v>
-      </c>
-      <c r="M5" s="3" t="s">
-        <v>43</v>
-      </c>
-      <c r="N5" s="3" t="str">
-        <f t="shared" si="1"/>
-        <v>累计出场 8 场</v>
-      </c>
-    </row>
-    <row r="6" ht="23" customHeight="1" spans="1:14">
-      <c r="A6" s="2">
-        <v>5</v>
-      </c>
-      <c r="B6" s="2" t="s">
-        <v>44</v>
-      </c>
-      <c r="C6" s="2" t="s">
-        <v>45</v>
-      </c>
-      <c r="D6" s="2">
-        <v>23</v>
-      </c>
-      <c r="E6" s="2" t="s">
-        <v>46</v>
-      </c>
-      <c r="F6" s="2" t="s">
-        <v>47</v>
-      </c>
-      <c r="G6" s="2">
-        <v>8</v>
-      </c>
-      <c r="H6" s="2">
-        <v>0</v>
-      </c>
-      <c r="I6" s="2">
-        <v>0</v>
-      </c>
-      <c r="J6" s="2">
-        <v>0</v>
-      </c>
-      <c r="K6" s="2">
-        <v>0</v>
-      </c>
-      <c r="L6" s="5">
-        <f t="shared" si="0"/>
-        <v>6.6</v>
-      </c>
-      <c r="M6" s="2" t="s">
-        <v>48</v>
-      </c>
-      <c r="N6" s="2" t="str">
-        <f t="shared" si="1"/>
-        <v>累计出场 8 场</v>
-      </c>
-    </row>
-    <row r="7" ht="23" customHeight="1" spans="1:14">
-      <c r="A7" s="3">
-        <v>6</v>
-      </c>
-      <c r="B7" s="3" t="s">
-        <v>49</v>
-      </c>
-      <c r="C7" s="3" t="s">
-        <v>50</v>
-      </c>
-      <c r="D7" s="3">
-        <v>9</v>
-      </c>
-      <c r="E7" s="3" t="s">
-        <v>29</v>
-      </c>
-      <c r="F7" s="3" t="s">
-        <v>51</v>
-      </c>
-      <c r="G7" s="3">
-        <v>0</v>
-      </c>
-      <c r="H7" s="3">
-        <v>0</v>
-      </c>
-      <c r="I7" s="3">
-        <v>0</v>
-      </c>
-      <c r="J7" s="3">
-        <v>0</v>
-      </c>
-      <c r="K7" s="3">
-        <v>0</v>
-      </c>
-      <c r="L7" s="6">
-        <f t="shared" si="0"/>
-        <v>6</v>
-      </c>
-      <c r="M7" s="3" t="s">
-        <v>52</v>
-      </c>
-      <c r="N7" s="3" t="str">
-        <f t="shared" si="1"/>
-        <v>累计出场 0 场</v>
-      </c>
-    </row>
-    <row r="8" ht="23" customHeight="1" spans="1:14">
-      <c r="A8" s="2">
-        <v>7</v>
-      </c>
-      <c r="B8" s="2" t="s">
+      <c r="N18" s="2" t="s">
         <v>53</v>
       </c>
-      <c r="C8" s="2" t="s">
-        <v>54</v>
-      </c>
-      <c r="D8" s="2">
-        <v>15</v>
-      </c>
-      <c r="E8" s="2" t="s">
-        <v>46</v>
-      </c>
-      <c r="F8" s="2" t="s">
-        <v>55</v>
-      </c>
-      <c r="G8" s="2">
-        <v>11</v>
-      </c>
-      <c r="H8" s="2">
-        <v>6</v>
-      </c>
-      <c r="I8" s="2">
-        <v>1</v>
-      </c>
-      <c r="J8" s="2">
-        <v>0</v>
-      </c>
-      <c r="K8" s="2">
-        <v>0</v>
-      </c>
-      <c r="L8" s="5">
-        <f t="shared" si="0"/>
-        <v>9.2</v>
-      </c>
-      <c r="M8" s="2" t="s">
-        <v>56</v>
-      </c>
-      <c r="N8" s="2" t="str">
-        <f t="shared" si="1"/>
-        <v>贡献 6 粒进球 / 送出 1 次助攻</v>
-      </c>
-    </row>
-    <row r="9" ht="23" customHeight="1" spans="1:14">
-      <c r="A9" s="3">
-        <v>8</v>
-      </c>
-      <c r="B9" s="3" t="s">
-        <v>57</v>
-      </c>
-      <c r="C9" s="3" t="s">
-        <v>58</v>
-      </c>
-      <c r="D9" s="3">
-        <v>8</v>
-      </c>
-      <c r="E9" s="3" t="s">
-        <v>59</v>
-      </c>
-      <c r="F9" s="3" t="s">
-        <v>60</v>
-      </c>
-      <c r="G9" s="3">
-        <v>8</v>
-      </c>
-      <c r="H9" s="3">
-        <v>2</v>
-      </c>
-      <c r="I9" s="3">
-        <v>3</v>
-      </c>
-      <c r="J9" s="3">
-        <v>0</v>
-      </c>
-      <c r="K9" s="3">
-        <v>0</v>
-      </c>
-      <c r="L9" s="6">
-        <f t="shared" si="0"/>
-        <v>8.1</v>
-      </c>
-      <c r="M9" s="3" t="s">
-        <v>61</v>
-      </c>
-      <c r="N9" s="3" t="str">
-        <f t="shared" si="1"/>
-        <v>贡献 2 粒进球 / 送出 3 次助攻</v>
-      </c>
-    </row>
-    <row r="10" ht="23" customHeight="1" spans="1:14">
-      <c r="A10" s="2">
-        <v>9</v>
-      </c>
-      <c r="B10" s="2" t="s">
-        <v>62</v>
-      </c>
-      <c r="C10" s="2" t="s">
-        <v>63</v>
-      </c>
-      <c r="D10" s="2">
-        <v>5</v>
-      </c>
-      <c r="E10" s="2" t="s">
-        <v>46</v>
-      </c>
-      <c r="F10" s="2" t="s">
-        <v>64</v>
-      </c>
-      <c r="G10" s="2">
-        <v>10</v>
-      </c>
-      <c r="H10" s="2">
-        <v>4</v>
-      </c>
-      <c r="I10" s="2">
-        <v>3</v>
-      </c>
-      <c r="J10" s="2">
-        <v>0</v>
-      </c>
-      <c r="K10" s="2">
-        <v>0</v>
-      </c>
-      <c r="L10" s="5">
-        <f t="shared" si="0"/>
-        <v>9</v>
-      </c>
-      <c r="M10" s="2" t="s">
-        <v>65</v>
-      </c>
-      <c r="N10" s="2" t="str">
-        <f t="shared" si="1"/>
-        <v>贡献 4 粒进球 / 送出 3 次助攻</v>
-      </c>
-    </row>
-    <row r="11" ht="23" customHeight="1" spans="1:14">
-      <c r="A11" s="3">
-        <v>10</v>
-      </c>
-      <c r="B11" s="3" t="s">
-        <v>66</v>
-      </c>
-      <c r="C11" s="3" t="s">
-        <v>67</v>
-      </c>
-      <c r="D11" s="3">
-        <v>17</v>
-      </c>
-      <c r="E11" s="3" t="s">
-        <v>29</v>
-      </c>
-      <c r="F11" s="3" t="s">
-        <v>30</v>
-      </c>
-      <c r="G11" s="3">
-        <v>6</v>
-      </c>
-      <c r="H11" s="3">
-        <v>0</v>
-      </c>
-      <c r="I11" s="3">
-        <v>0</v>
-      </c>
-      <c r="J11" s="3">
-        <v>0</v>
-      </c>
-      <c r="K11" s="3">
-        <v>0</v>
-      </c>
-      <c r="L11" s="6">
-        <f t="shared" si="0"/>
-        <v>6.5</v>
-      </c>
-      <c r="M11" s="3" t="s">
-        <v>68</v>
-      </c>
-      <c r="N11" s="3" t="str">
-        <f t="shared" si="1"/>
-        <v>累计出场 6 场</v>
-      </c>
-    </row>
-    <row r="12" ht="23" customHeight="1" spans="1:14">
-      <c r="A12" s="2">
-        <v>11</v>
-      </c>
-      <c r="B12" s="2" t="s">
-        <v>69</v>
-      </c>
-      <c r="C12" s="2" t="s">
-        <v>41</v>
-      </c>
-      <c r="D12" s="2">
-        <v>18</v>
-      </c>
-      <c r="E12" s="2" t="s">
-        <v>42</v>
-      </c>
-      <c r="F12" s="2" t="s">
-        <v>70</v>
-      </c>
-      <c r="G12" s="2">
-        <v>5</v>
-      </c>
-      <c r="H12" s="2">
-        <v>0</v>
-      </c>
-      <c r="I12" s="2">
-        <v>0</v>
-      </c>
-      <c r="J12" s="2">
-        <v>0</v>
-      </c>
-      <c r="K12" s="2">
-        <v>1</v>
-      </c>
-      <c r="L12" s="5">
-        <f t="shared" si="0"/>
-        <v>6.6</v>
-      </c>
-      <c r="M12" s="2" t="s">
-        <v>43</v>
-      </c>
-      <c r="N12" s="2" t="str">
-        <f t="shared" si="1"/>
-        <v>累计出场 5 场</v>
-      </c>
-    </row>
-    <row r="13" ht="23" customHeight="1" spans="1:14">
-      <c r="A13" s="3">
-        <v>12</v>
-      </c>
-      <c r="B13" s="3" t="s">
-        <v>71</v>
-      </c>
-      <c r="C13" s="3" t="s">
-        <v>72</v>
-      </c>
-      <c r="D13" s="3">
-        <v>19</v>
-      </c>
-      <c r="E13" s="3" t="s">
-        <v>29</v>
-      </c>
-      <c r="F13" s="3" t="s">
-        <v>51</v>
-      </c>
-      <c r="G13" s="3">
-        <v>8</v>
-      </c>
-      <c r="H13" s="3">
-        <v>0</v>
-      </c>
-      <c r="I13" s="3">
-        <v>0</v>
-      </c>
-      <c r="J13" s="3">
-        <v>0</v>
-      </c>
-      <c r="K13" s="3">
-        <v>0</v>
-      </c>
-      <c r="L13" s="6">
-        <f t="shared" si="0"/>
-        <v>6.6</v>
-      </c>
-      <c r="M13" s="3" t="s">
-        <v>73</v>
-      </c>
-      <c r="N13" s="3" t="str">
-        <f t="shared" si="1"/>
-        <v>累计出场 8 场</v>
-      </c>
-    </row>
-    <row r="14" ht="23" customHeight="1" spans="1:14">
-      <c r="A14" s="2">
-        <v>13</v>
-      </c>
-      <c r="B14" s="2" t="s">
-        <v>74</v>
-      </c>
-      <c r="C14" s="2" t="s">
-        <v>75</v>
-      </c>
-      <c r="D14" s="2">
-        <v>25</v>
-      </c>
-      <c r="E14" s="2" t="s">
-        <v>59</v>
-      </c>
-      <c r="F14" s="2" t="s">
-        <v>76</v>
-      </c>
-      <c r="G14" s="2">
-        <v>6</v>
-      </c>
-      <c r="H14" s="2">
-        <v>0</v>
-      </c>
-      <c r="I14" s="2">
-        <v>0</v>
-      </c>
-      <c r="J14" s="2">
-        <v>0</v>
-      </c>
-      <c r="K14" s="2">
-        <v>0</v>
-      </c>
-      <c r="L14" s="5">
-        <f t="shared" si="0"/>
-        <v>6.5</v>
-      </c>
-      <c r="M14" s="2" t="s">
-        <v>68</v>
-      </c>
-      <c r="N14" s="2" t="str">
-        <f t="shared" si="1"/>
-        <v>累计出场 6 场</v>
-      </c>
-    </row>
-    <row r="15" ht="23" customHeight="1" spans="1:14">
-      <c r="A15" s="3">
-        <v>14</v>
-      </c>
-      <c r="B15" s="3" t="s">
-        <v>77</v>
-      </c>
-      <c r="C15" s="3" t="s">
-        <v>78</v>
-      </c>
-      <c r="D15" s="3">
-        <v>66</v>
-      </c>
-      <c r="E15" s="3" t="s">
-        <v>29</v>
-      </c>
-      <c r="F15" s="3" t="s">
-        <v>79</v>
-      </c>
-      <c r="G15" s="3">
-        <v>3</v>
-      </c>
-      <c r="H15" s="3">
-        <v>0</v>
-      </c>
-      <c r="I15" s="3">
-        <v>0</v>
-      </c>
-      <c r="J15" s="3">
-        <v>0</v>
-      </c>
-      <c r="K15" s="3">
-        <v>0</v>
-      </c>
-      <c r="L15" s="6">
-        <f t="shared" si="0"/>
-        <v>6.2</v>
-      </c>
-      <c r="M15" s="3" t="s">
-        <v>52</v>
-      </c>
-      <c r="N15" s="3" t="str">
-        <f t="shared" si="1"/>
-        <v>累计出场 3 场</v>
-      </c>
-    </row>
-    <row r="16" ht="23" customHeight="1" spans="1:14">
-      <c r="A16" s="2">
-        <v>15</v>
-      </c>
-      <c r="B16" s="2" t="s">
-        <v>80</v>
-      </c>
-      <c r="C16" s="2" t="s">
-        <v>81</v>
-      </c>
-      <c r="D16" s="2">
-        <v>12</v>
-      </c>
-      <c r="E16" s="2" t="s">
-        <v>59</v>
-      </c>
-      <c r="F16" s="2" t="s">
-        <v>82</v>
-      </c>
-      <c r="G16" s="2">
-        <v>10</v>
-      </c>
-      <c r="H16" s="2">
-        <v>1</v>
-      </c>
-      <c r="I16" s="2">
-        <v>1</v>
-      </c>
-      <c r="J16" s="2">
-        <v>0</v>
-      </c>
-      <c r="K16" s="2">
-        <v>1</v>
-      </c>
-      <c r="L16" s="5">
-        <f t="shared" si="0"/>
-        <v>7.6</v>
-      </c>
-      <c r="M16" s="2" t="s">
-        <v>83</v>
-      </c>
-      <c r="N16" s="2" t="str">
-        <f t="shared" si="1"/>
-        <v>贡献 1 粒进球 / 送出 1 次助攻</v>
-      </c>
-    </row>
-    <row r="17" ht="23" customHeight="1" spans="1:14">
-      <c r="A17" s="3">
-        <v>16</v>
-      </c>
-      <c r="B17" s="3" t="s">
-        <v>84</v>
-      </c>
-      <c r="C17" s="3" t="s">
-        <v>85</v>
-      </c>
-      <c r="D17" s="3">
-        <v>66</v>
-      </c>
-      <c r="E17" s="3" t="s">
-        <v>42</v>
-      </c>
-      <c r="F17" s="3" t="s">
-        <v>42</v>
-      </c>
-      <c r="G17" s="3">
-        <v>1</v>
-      </c>
-      <c r="H17" s="3">
-        <v>0</v>
-      </c>
-      <c r="I17" s="3">
-        <v>0</v>
-      </c>
-      <c r="J17" s="3">
-        <v>0</v>
-      </c>
-      <c r="K17" s="3">
-        <v>0</v>
-      </c>
-      <c r="L17" s="6">
-        <f t="shared" si="0"/>
-        <v>6.1</v>
-      </c>
-      <c r="M17" s="3" t="s">
-        <v>86</v>
-      </c>
-      <c r="N17" s="3" t="str">
-        <f t="shared" si="1"/>
-        <v>累计出场 1 场</v>
-      </c>
-    </row>
-    <row r="18" ht="23" customHeight="1" spans="1:14">
-      <c r="A18" s="2">
-        <v>17</v>
-      </c>
-      <c r="B18" s="2" t="s">
-        <v>87</v>
-      </c>
-      <c r="C18" s="2" t="s">
-        <v>88</v>
-      </c>
-      <c r="D18" s="2">
-        <v>15</v>
-      </c>
-      <c r="E18" s="2" t="s">
-        <v>29</v>
-      </c>
-      <c r="F18" s="2" t="s">
-        <v>89</v>
-      </c>
-      <c r="G18" s="2">
-        <v>2</v>
-      </c>
-      <c r="H18" s="2">
-        <v>0</v>
-      </c>
-      <c r="I18" s="2">
-        <v>0</v>
-      </c>
-      <c r="J18" s="2">
-        <v>0</v>
-      </c>
-      <c r="K18" s="2">
-        <v>0</v>
-      </c>
-      <c r="L18" s="5">
-        <f t="shared" si="0"/>
-        <v>6.2</v>
-      </c>
-      <c r="M18" s="2" t="s">
-        <v>52</v>
-      </c>
-      <c r="N18" s="2" t="str">
+      <c r="O18" s="2" t="str">
         <f t="shared" si="1"/>
         <v>累计出场 2 场</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData" ref="A1:N18" etc:filterBottomFollowUsedRange="0">
+  <autoFilter xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData" ref="A1:O18" etc:filterBottomFollowUsedRange="0">
     <extLst/>
   </autoFilter>
   <conditionalFormatting sqref="M2:M18">
@@ -2595,82 +2653,82 @@
   <sheetData>
     <row r="1" ht="26" customHeight="1" spans="1:6">
       <c r="A1" s="1" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>91</v>
+        <v>92</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>92</v>
+        <v>93</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>93</v>
+        <v>94</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>94</v>
+        <v>95</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
     </row>
     <row r="2" ht="27" customHeight="1" spans="1:6">
       <c r="A2" s="2" t="s">
-        <v>96</v>
+        <v>97</v>
       </c>
       <c r="B2" s="2" t="s">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="C2" s="2" t="s">
-        <v>98</v>
+        <v>99</v>
       </c>
       <c r="D2" s="2" t="s">
-        <v>98</v>
+        <v>99</v>
       </c>
       <c r="E2" s="2" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="F2" s="2" t="s">
-        <v>100</v>
+        <v>101</v>
       </c>
     </row>
     <row r="3" ht="27" customHeight="1" spans="1:6">
       <c r="A3" s="3" t="s">
-        <v>101</v>
+        <v>102</v>
       </c>
       <c r="B3" s="3" t="s">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="C3" s="3" t="s">
-        <v>102</v>
+        <v>103</v>
       </c>
       <c r="D3" s="3" t="s">
-        <v>102</v>
+        <v>103</v>
       </c>
       <c r="E3" s="3" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="F3" s="3" t="s">
-        <v>104</v>
+        <v>105</v>
       </c>
     </row>
     <row r="4" spans="1:6">
       <c r="A4" s="2" t="s">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="B4" s="2" t="s">
-        <v>106</v>
+        <v>107</v>
       </c>
       <c r="C4" s="2" t="s">
-        <v>107</v>
+        <v>108</v>
       </c>
       <c r="D4" s="2" t="s">
-        <v>107</v>
+        <v>108</v>
       </c>
       <c r="E4" s="2" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="F4" s="2" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
     </row>
   </sheetData>
@@ -2701,350 +2759,350 @@
   <sheetData>
     <row r="1" ht="26" customHeight="1" spans="1:9">
       <c r="A1" s="1" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>92</v>
+        <v>93</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>111</v>
+        <v>112</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>112</v>
+        <v>113</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>113</v>
+        <v>114</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>114</v>
+        <v>115</v>
       </c>
       <c r="G1" s="1" t="s">
-        <v>115</v>
+        <v>116</v>
       </c>
       <c r="H1" s="1" t="s">
-        <v>116</v>
+        <v>117</v>
       </c>
       <c r="I1" s="1" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
     </row>
     <row r="2" spans="1:9">
       <c r="A2" s="2" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="B2" s="2" t="s">
-        <v>107</v>
+        <v>108</v>
       </c>
       <c r="C2" s="2" t="s">
-        <v>119</v>
+        <v>120</v>
       </c>
       <c r="D2" s="2" t="s">
-        <v>120</v>
+        <v>121</v>
       </c>
       <c r="E2" s="2" t="s">
-        <v>121</v>
+        <v>122</v>
       </c>
       <c r="F2" s="2" t="s">
-        <v>122</v>
+        <v>123</v>
       </c>
       <c r="G2" s="2" t="s">
-        <v>123</v>
+        <v>124</v>
       </c>
       <c r="H2" s="2" t="s">
-        <v>124</v>
+        <v>125</v>
       </c>
       <c r="I2" s="2" t="s">
-        <v>125</v>
+        <v>126</v>
       </c>
     </row>
     <row r="3" spans="1:9">
       <c r="A3" s="3" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="B3" s="3" t="s">
-        <v>107</v>
+        <v>108</v>
       </c>
       <c r="C3" s="3" t="s">
-        <v>126</v>
+        <v>127</v>
       </c>
       <c r="D3" s="3" t="s">
-        <v>127</v>
+        <v>128</v>
       </c>
       <c r="E3" s="3" t="s">
-        <v>128</v>
+        <v>129</v>
       </c>
       <c r="F3" s="3" t="s">
-        <v>122</v>
+        <v>123</v>
       </c>
       <c r="G3" s="3" t="s">
-        <v>123</v>
+        <v>124</v>
       </c>
       <c r="H3" s="3" t="s">
-        <v>129</v>
+        <v>130</v>
       </c>
       <c r="I3" s="3" t="s">
-        <v>130</v>
+        <v>131</v>
       </c>
     </row>
     <row r="4" spans="1:9">
       <c r="A4" s="2" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="B4" s="2" t="s">
-        <v>107</v>
+        <v>108</v>
       </c>
       <c r="C4" s="2" t="s">
-        <v>131</v>
+        <v>132</v>
       </c>
       <c r="D4" s="2" t="s">
-        <v>132</v>
+        <v>133</v>
       </c>
       <c r="E4" s="2" t="s">
-        <v>133</v>
+        <v>134</v>
       </c>
       <c r="F4" s="2" t="s">
-        <v>122</v>
+        <v>123</v>
       </c>
       <c r="G4" s="2" t="s">
-        <v>123</v>
+        <v>124</v>
       </c>
       <c r="H4" s="2" t="s">
-        <v>134</v>
+        <v>135</v>
       </c>
       <c r="I4" s="2" t="s">
-        <v>135</v>
+        <v>136</v>
       </c>
     </row>
     <row r="5" ht="27" customHeight="1" spans="1:9">
       <c r="A5" s="3" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="B5" s="3" t="s">
-        <v>102</v>
+        <v>103</v>
       </c>
       <c r="C5" s="3" t="s">
-        <v>136</v>
+        <v>137</v>
       </c>
       <c r="D5" s="3" t="s">
-        <v>132</v>
+        <v>133</v>
       </c>
       <c r="E5" s="3" t="s">
-        <v>137</v>
+        <v>138</v>
       </c>
       <c r="F5" s="3" t="s">
-        <v>138</v>
+        <v>139</v>
       </c>
       <c r="G5" s="3" t="s">
-        <v>123</v>
+        <v>124</v>
       </c>
       <c r="H5" s="3" t="s">
-        <v>139</v>
+        <v>140</v>
       </c>
       <c r="I5" s="3" t="s">
-        <v>140</v>
+        <v>141</v>
       </c>
     </row>
     <row r="6" spans="1:9">
       <c r="A6" s="2" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="B6" s="2" t="s">
-        <v>102</v>
+        <v>103</v>
       </c>
       <c r="C6" s="2" t="s">
-        <v>141</v>
+        <v>142</v>
       </c>
       <c r="D6" s="2" t="s">
-        <v>142</v>
+        <v>143</v>
       </c>
       <c r="E6" s="2" t="s">
-        <v>143</v>
+        <v>144</v>
       </c>
       <c r="F6" s="2" t="s">
-        <v>122</v>
+        <v>123</v>
       </c>
       <c r="G6" s="2" t="s">
-        <v>123</v>
+        <v>124</v>
       </c>
       <c r="H6" s="2" t="s">
-        <v>124</v>
+        <v>125</v>
       </c>
       <c r="I6" s="2" t="s">
-        <v>144</v>
+        <v>145</v>
       </c>
     </row>
     <row r="7" spans="1:9">
       <c r="A7" s="3" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="B7" s="3" t="s">
-        <v>102</v>
+        <v>103</v>
       </c>
       <c r="C7" s="3" t="s">
-        <v>145</v>
+        <v>146</v>
       </c>
       <c r="D7" s="3" t="s">
-        <v>146</v>
+        <v>147</v>
       </c>
       <c r="E7" s="3" t="s">
-        <v>147</v>
+        <v>148</v>
       </c>
       <c r="F7" s="3" t="s">
-        <v>122</v>
+        <v>123</v>
       </c>
       <c r="G7" s="3" t="s">
-        <v>123</v>
+        <v>124</v>
       </c>
       <c r="H7" s="3" t="s">
-        <v>148</v>
+        <v>149</v>
       </c>
       <c r="I7" s="3" t="s">
-        <v>149</v>
+        <v>150</v>
       </c>
     </row>
     <row r="8" spans="1:9">
       <c r="A8" s="2" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="B8" s="2" t="s">
-        <v>102</v>
+        <v>103</v>
       </c>
       <c r="C8" s="2" t="s">
-        <v>150</v>
+        <v>151</v>
       </c>
       <c r="D8" s="2" t="s">
-        <v>151</v>
+        <v>152</v>
       </c>
       <c r="E8" s="2" t="s">
-        <v>152</v>
+        <v>153</v>
       </c>
       <c r="F8" s="2" t="s">
-        <v>138</v>
+        <v>139</v>
       </c>
       <c r="G8" s="2" t="s">
-        <v>123</v>
+        <v>124</v>
       </c>
       <c r="H8" s="2" t="s">
-        <v>153</v>
+        <v>154</v>
       </c>
       <c r="I8" s="2" t="s">
-        <v>154</v>
+        <v>155</v>
       </c>
     </row>
     <row r="9" spans="1:9">
       <c r="A9" s="3" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="B9" s="3" t="s">
-        <v>102</v>
+        <v>103</v>
       </c>
       <c r="C9" s="3" t="s">
-        <v>155</v>
+        <v>156</v>
       </c>
       <c r="D9" s="3" t="s">
-        <v>156</v>
+        <v>157</v>
       </c>
       <c r="E9" s="3" t="s">
-        <v>137</v>
+        <v>138</v>
       </c>
       <c r="F9" s="3" t="s">
-        <v>138</v>
+        <v>139</v>
       </c>
       <c r="G9" s="3" t="s">
-        <v>123</v>
+        <v>124</v>
       </c>
       <c r="H9" s="3" t="s">
-        <v>157</v>
+        <v>158</v>
       </c>
       <c r="I9" s="3" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
     </row>
     <row r="10" spans="1:9">
       <c r="A10" s="2" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="B10" s="2" t="s">
-        <v>102</v>
+        <v>103</v>
       </c>
       <c r="C10" s="2" t="s">
-        <v>159</v>
+        <v>160</v>
       </c>
       <c r="D10" s="2" t="s">
-        <v>160</v>
+        <v>161</v>
       </c>
       <c r="E10" s="2" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
       <c r="F10" s="2" t="s">
-        <v>122</v>
+        <v>123</v>
       </c>
       <c r="G10" s="2" t="s">
-        <v>123</v>
+        <v>124</v>
       </c>
       <c r="H10" s="2" t="s">
-        <v>124</v>
+        <v>125</v>
       </c>
       <c r="I10" s="2" t="s">
-        <v>162</v>
+        <v>163</v>
       </c>
     </row>
     <row r="11" spans="1:9">
       <c r="A11" s="3" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="B11" s="3" t="s">
-        <v>98</v>
+        <v>99</v>
       </c>
       <c r="C11" s="3" t="s">
-        <v>163</v>
+        <v>164</v>
       </c>
       <c r="D11" s="3" t="s">
-        <v>120</v>
+        <v>121</v>
       </c>
       <c r="E11" s="3" t="s">
-        <v>164</v>
+        <v>165</v>
       </c>
       <c r="F11" s="3" t="s">
-        <v>122</v>
+        <v>123</v>
       </c>
       <c r="G11" s="3" t="s">
-        <v>123</v>
+        <v>124</v>
       </c>
       <c r="H11" s="3" t="s">
-        <v>165</v>
+        <v>166</v>
       </c>
       <c r="I11" s="3" t="s">
-        <v>166</v>
+        <v>167</v>
       </c>
     </row>
     <row r="12" ht="27" customHeight="1" spans="1:9">
       <c r="A12" s="2" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="B12" s="2" t="s">
-        <v>98</v>
+        <v>99</v>
       </c>
       <c r="C12" s="2" t="s">
-        <v>167</v>
+        <v>168</v>
       </c>
       <c r="D12" s="2" t="s">
-        <v>132</v>
+        <v>133</v>
       </c>
       <c r="E12" s="2" t="s">
-        <v>168</v>
+        <v>169</v>
       </c>
       <c r="F12" s="2" t="s">
-        <v>122</v>
+        <v>123</v>
       </c>
       <c r="G12" s="2" t="s">
-        <v>123</v>
+        <v>124</v>
       </c>
       <c r="H12" s="2" t="s">
-        <v>169</v>
+        <v>170</v>
       </c>
       <c r="I12" s="2" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Add isolated newcomer data pipeline
</commit_message>
<xml_diff>
--- a/data/生康足球队数据源.xlsx
+++ b/data/生康足球队数据源.xlsx
@@ -11,11 +11,13 @@
     <sheet name="球员数据" sheetId="2" r:id="rId2"/>
     <sheet name="赛事索引" sheetId="3" r:id="rId3"/>
     <sheet name="赛程" sheetId="4" r:id="rId4"/>
+    <sheet name="新生展示" sheetId="5" r:id="rId5"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">球员数据!$A$1:$O$18</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">赛事索引!$A$1:$F$4</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">赛程!$A$1:$I$12</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">新生展示!$A$1:$L$1</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
@@ -35,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="245" uniqueCount="172">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="257" uniqueCount="179">
   <si>
     <t>生康足球队 · 球员数据汇总</t>
   </si>
@@ -551,6 +553,27 @@
   </si>
   <si>
     <t>球队十一人制正式首战，雨中作战，比分并非一边倒。</t>
+  </si>
+  <si>
+    <t>排序</t>
+  </si>
+  <si>
+    <t>年级</t>
+  </si>
+  <si>
+    <t>惯用脚</t>
+  </si>
+  <si>
+    <t>自我介绍</t>
+  </si>
+  <si>
+    <t>照片文件名</t>
+  </si>
+  <si>
+    <t>照片焦点</t>
+  </si>
+  <si>
+    <t>展示状态</t>
   </si>
 </sst>
 </file>
@@ -3112,4 +3135,71 @@
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <headerFooter/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
+  <sheetPr/>
+  <dimension ref="A1:L1"/>
+  <sheetFormatPr defaultColWidth="9" defaultRowHeight="13.5"/>
+  <cols>
+    <col min="1" max="1" width="8" customWidth="1"/>
+    <col min="2" max="2" width="12" customWidth="1"/>
+    <col min="3" max="3" width="10" customWidth="1"/>
+    <col min="4" max="4" width="8" customWidth="1"/>
+    <col min="5" max="5" width="10" customWidth="1"/>
+    <col min="6" max="6" width="18" customWidth="1"/>
+    <col min="7" max="7" width="10" customWidth="1"/>
+    <col min="8" max="8" width="18" customWidth="1"/>
+    <col min="9" max="9" width="34" customWidth="1"/>
+    <col min="10" max="10" width="24" customWidth="1"/>
+    <col min="11" max="11" width="14" customWidth="1"/>
+    <col min="12" max="12" width="12" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="26" customHeight="1" spans="1:12">
+      <c r="A1" s="1" t="s">
+        <v>172</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>173</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>16</v>
+      </c>
+      <c r="E1" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="F1" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="G1" s="1" t="s">
+        <v>174</v>
+      </c>
+      <c r="H1" s="1" t="s">
+        <v>26</v>
+      </c>
+      <c r="I1" s="1" t="s">
+        <v>175</v>
+      </c>
+      <c r="J1" s="1" t="s">
+        <v>176</v>
+      </c>
+      <c r="K1" s="1" t="s">
+        <v>177</v>
+      </c>
+      <c r="L1" s="1" t="s">
+        <v>178</v>
+      </c>
+    </row>
+  </sheetData>
+  <autoFilter xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData" ref="A1:L1" etc:filterBottomFollowUsedRange="0">
+    <extLst/>
+  </autoFilter>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <headerFooter/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
Fix newcomer final review findings
</commit_message>
<xml_diff>
--- a/data/生康足球队数据源.xlsx
+++ b/data/生康足球队数据源.xlsx
@@ -1264,132 +1264,132 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:D8"/>
-  <sheetFormatPr baseColWidth="8" defaultColWidth="9" defaultRowHeight="13.5" outlineLevelRow="7"/>
-  <cols>
-    <col width="16" customWidth="1" min="1" max="1"/>
-    <col width="22" customWidth="1" min="2" max="2"/>
-    <col width="4" customWidth="1" min="3" max="3"/>
-    <col width="46" customWidth="1" min="4" max="4"/>
-  </cols>
-  <sheetData>
-    <row r="1" ht="32" customHeight="1">
-      <c r="A1" s="7" t="inlineStr">
-        <is>
-          <t>生康足球队 · 球员数据汇总</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" s="8" t="inlineStr">
-        <is>
-          <t>数据范围</t>
-        </is>
-      </c>
-      <c r="B3" s="2" t="inlineStr">
-        <is>
-          <t>网站当前球员档案</t>
-        </is>
-      </c>
-      <c r="C3" s="2" t="n"/>
-      <c r="D3" s="8" t="inlineStr">
-        <is>
-          <t>说明</t>
-        </is>
-      </c>
-    </row>
-    <row r="4" ht="15" customHeight="1">
-      <c r="A4" s="9" t="inlineStr">
-        <is>
-          <t>球员人数</t>
-        </is>
-      </c>
-      <c r="B4" s="10">
-        <f>COUNTA(球员数据!B2:B18)</f>
-        <v/>
-      </c>
-      <c r="C4" s="3" t="n"/>
-      <c r="D4" s="3" t="inlineStr">
-        <is>
-          <t>数据来源：网站 js/team-data.js</t>
-        </is>
-      </c>
-    </row>
-    <row r="5" ht="15" customHeight="1">
-      <c r="A5" s="8" t="inlineStr">
-        <is>
-          <t>总出场</t>
-        </is>
-      </c>
-      <c r="B5" s="11">
-        <f>SUM(球员数据!G2:G18)</f>
-        <v/>
-      </c>
-      <c r="C5" s="2" t="n"/>
-      <c r="D5" s="2" t="inlineStr">
-        <is>
-          <t>评分为网站现有记录，不做额外计算。</t>
-        </is>
-      </c>
-    </row>
-    <row r="6" ht="15" customHeight="1">
-      <c r="A6" s="9" t="inlineStr">
-        <is>
-          <t>总进球</t>
-        </is>
-      </c>
-      <c r="B6" s="10">
-        <f>SUM(球员数据!H2:H18)</f>
-        <v/>
-      </c>
-      <c r="C6" s="3" t="n"/>
-      <c r="D6" s="3" t="inlineStr">
-        <is>
-          <t>扑救与零封字段保留，当前未统计时为 0。</t>
-        </is>
-      </c>
-    </row>
-    <row r="7" ht="15" customHeight="1">
-      <c r="A7" s="8" t="inlineStr">
-        <is>
-          <t>总助攻</t>
-        </is>
-      </c>
-      <c r="B7" s="11">
-        <f>SUM(球员数据!I2:I18)</f>
-        <v/>
-      </c>
-      <c r="C7" s="2" t="n"/>
-      <c r="D7" s="2" t="inlineStr">
-        <is>
-          <t>后续只需更新“球员数据”工作表或网站源数据。</t>
-        </is>
-      </c>
-    </row>
-    <row r="8" ht="15" customHeight="1">
-      <c r="A8" s="9" t="inlineStr">
-        <is>
-          <t>总 MVP</t>
-        </is>
-      </c>
-      <c r="B8" s="10">
-        <f>SUM(球员数据!J2:J18)</f>
-        <v/>
-      </c>
-      <c r="C8" s="3" t="n"/>
-      <c r="D8" s="3" t="n"/>
-    </row>
-  </sheetData>
-  <mergeCells count="1">
-    <mergeCell ref="A1:D1"/>
-  </mergeCells>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
+<s:worksheet xmlns:s="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <s:sheetPr>
+    <s:outlinePr summaryBelow="1" summaryRight="1"/>
+    <s:pageSetUpPr/>
+  </s:sheetPr>
+  <s:dimension ref="A1:D8"/>
+  <s:sheetFormatPr baseColWidth="8" defaultColWidth="9" defaultRowHeight="13.5" outlineLevelRow="7"/>
+  <s:cols>
+    <s:col width="16" customWidth="1" min="1" max="1"/>
+    <s:col width="22" customWidth="1" min="2" max="2"/>
+    <s:col width="4" customWidth="1" min="3" max="3"/>
+    <s:col width="46" customWidth="1" min="4" max="4"/>
+  </s:cols>
+  <s:sheetData>
+    <s:row r="1" ht="32" customHeight="1">
+      <s:c r="A1" s="7" t="inlineStr">
+        <s:is>
+          <s:t>生康足球队 · 球员数据汇总</s:t>
+        </s:is>
+      </s:c>
+    </s:row>
+    <s:row r="3">
+      <s:c r="A3" s="8" t="inlineStr">
+        <s:is>
+          <s:t>数据范围</s:t>
+        </s:is>
+      </s:c>
+      <s:c r="B3" s="2" t="inlineStr">
+        <s:is>
+          <s:t>网站当前球员档案</s:t>
+        </s:is>
+      </s:c>
+      <s:c r="C3" s="2" t="n"/>
+      <s:c r="D3" s="8" t="inlineStr">
+        <s:is>
+          <s:t>说明</s:t>
+        </s:is>
+      </s:c>
+    </s:row>
+    <s:row r="4" ht="15" customHeight="1">
+      <s:c r="A4" s="9" t="inlineStr">
+        <s:is>
+          <s:t>球员人数</s:t>
+        </s:is>
+      </s:c>
+      <s:c r="B4" s="10">
+        <s:f>COUNTA(球员数据!B2:B18)</s:f>
+        <s:v>17</s:v>
+      </s:c>
+      <s:c r="C4" s="3" t="n"/>
+      <s:c r="D4" s="3" t="inlineStr">
+        <s:is>
+          <s:t>数据来源：网站 js/team-data.js</s:t>
+        </s:is>
+      </s:c>
+    </s:row>
+    <s:row r="5" ht="15" customHeight="1">
+      <s:c r="A5" s="8" t="inlineStr">
+        <s:is>
+          <s:t>总出场</s:t>
+        </s:is>
+      </s:c>
+      <s:c r="B5" s="11">
+        <s:f>SUM(球员数据!G2:G18)</s:f>
+        <s:v>110</s:v>
+      </s:c>
+      <s:c r="C5" s="2" t="n"/>
+      <s:c r="D5" s="2" t="inlineStr">
+        <s:is>
+          <s:t>评分为网站现有记录，不做额外计算。</s:t>
+        </s:is>
+      </s:c>
+    </s:row>
+    <s:row r="6" ht="15" customHeight="1">
+      <s:c r="A6" s="9" t="inlineStr">
+        <s:is>
+          <s:t>总进球</s:t>
+        </s:is>
+      </s:c>
+      <s:c r="B6" s="10">
+        <s:f>SUM(球员数据!H2:H18)</s:f>
+        <s:v>13</s:v>
+      </s:c>
+      <s:c r="C6" s="3" t="n"/>
+      <s:c r="D6" s="3" t="inlineStr">
+        <s:is>
+          <s:t>扑救与零封字段保留，当前未统计时为 0。</s:t>
+        </s:is>
+      </s:c>
+    </s:row>
+    <s:row r="7" ht="15" customHeight="1">
+      <s:c r="A7" s="8" t="inlineStr">
+        <s:is>
+          <s:t>总助攻</s:t>
+        </s:is>
+      </s:c>
+      <s:c r="B7" s="11">
+        <s:f>SUM(球员数据!I2:I18)</s:f>
+        <s:v>9</s:v>
+      </s:c>
+      <s:c r="C7" s="2" t="n"/>
+      <s:c r="D7" s="2" t="inlineStr">
+        <s:is>
+          <s:t>后续只需更新“球员数据”工作表或网站源数据。</s:t>
+        </s:is>
+      </s:c>
+    </s:row>
+    <s:row r="8" ht="15" customHeight="1">
+      <s:c r="A8" s="9" t="inlineStr">
+        <s:is>
+          <s:t>总 MVP</s:t>
+        </s:is>
+      </s:c>
+      <s:c r="B8" s="10">
+        <s:f>SUM(球员数据!J2:J18)</s:f>
+        <s:v>0</s:v>
+      </s:c>
+      <s:c r="C8" s="3" t="n"/>
+      <s:c r="D8" s="3" t="n"/>
+    </s:row>
+  </s:sheetData>
+  <s:mergeCells count="1">
+    <s:mergeCell ref="A1:D1"/>
+  </s:mergeCells>
+  <s:pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</s:worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>

</xml_diff>

<commit_message>
Add isolated team manager data source
</commit_message>
<xml_diff>
--- a/data/生康足球队数据源.xlsx
+++ b/data/生康足球队数据源.xlsx
@@ -11,12 +11,14 @@
     <sheet name="赛事索引" sheetId="3" state="visible" r:id="rId3"/>
     <sheet name="赛程" sheetId="4" state="visible" r:id="rId4"/>
     <sheet name="新生展示" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="球队经理" sheetId="6" state="visible" r:id="rId6"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'球员数据'!$A$1:$O$18</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'赛事索引'!$A$1:$F$4</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'赛程'!$A$1:$I$12</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'新生展示'!$A$1:$L$1</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'球队经理'!$A$1:$J$1</definedName>
   </definedNames>
   <calcPr calcId="191029" fullCalcOnLoad="1" forceFullCalc="1"/>
 </workbook>
@@ -976,6 +978,25 @@
     <tableColumn id="10" name="照片文件名"/>
     <tableColumn id="11" name="照片焦点"/>
     <tableColumn id="12" name="展示状态"/>
+  </tableColumns>
+  <tableStyleInfo name="TableStyleMedium4" showFirstColumn="0" showLastColumn="0" showRowStripes="0" showColumnStripes="0"/>
+</table>
+</file>
+
+<file path=xl/tables/table5.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="5" name="TeamManagers" displayName="TeamManagers" ref="A1:J1" headerRowCount="1">
+  <autoFilter ref="A1:J1"/>
+  <tableColumns count="10">
+    <tableColumn id="1" name="排序"/>
+    <tableColumn id="2" name="姓名"/>
+    <tableColumn id="3" name="年级"/>
+    <tableColumn id="4" name="加入赛季"/>
+    <tableColumn id="5" name="身份"/>
+    <tableColumn id="6" name="职责"/>
+    <tableColumn id="7" name="个人介绍"/>
+    <tableColumn id="8" name="照片文件名"/>
+    <tableColumn id="9" name="照片焦点"/>
+    <tableColumn id="10" name="展示状态"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium4" showFirstColumn="0" showLastColumn="0" showRowStripes="0" showColumnStripes="0"/>
 </table>
@@ -3358,4 +3379,86 @@
     <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
   </tableParts>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:J1"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="8" customWidth="1" min="1" max="1"/>
+    <col width="12" customWidth="1" min="2" max="2"/>
+    <col width="10" customWidth="1" min="3" max="3"/>
+    <col width="14" customWidth="1" min="4" max="4"/>
+    <col width="14" customWidth="1" min="5" max="5"/>
+    <col width="46" customWidth="1" min="6" max="6"/>
+    <col width="38" customWidth="1" min="7" max="7"/>
+    <col width="26" customWidth="1" min="8" max="8"/>
+    <col width="14" customWidth="1" min="9" max="9"/>
+    <col width="12" customWidth="1" min="10" max="10"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="26" customHeight="1">
+      <c r="A1" s="13" t="inlineStr">
+        <is>
+          <t>排序</t>
+        </is>
+      </c>
+      <c r="B1" s="13" t="inlineStr">
+        <is>
+          <t>姓名</t>
+        </is>
+      </c>
+      <c r="C1" s="13" t="inlineStr">
+        <is>
+          <t>年级</t>
+        </is>
+      </c>
+      <c r="D1" s="13" t="inlineStr">
+        <is>
+          <t>加入赛季</t>
+        </is>
+      </c>
+      <c r="E1" s="13" t="inlineStr">
+        <is>
+          <t>身份</t>
+        </is>
+      </c>
+      <c r="F1" s="13" t="inlineStr">
+        <is>
+          <t>职责</t>
+        </is>
+      </c>
+      <c r="G1" s="13" t="inlineStr">
+        <is>
+          <t>个人介绍</t>
+        </is>
+      </c>
+      <c r="H1" s="13" t="inlineStr">
+        <is>
+          <t>照片文件名</t>
+        </is>
+      </c>
+      <c r="I1" s="13" t="inlineStr">
+        <is>
+          <t>照片焦点</t>
+        </is>
+      </c>
+      <c r="J1" s="13" t="inlineStr">
+        <is>
+          <t>展示状态</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <autoFilter ref="A1:J1"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <tableParts count="1">
+    <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
+  </tableParts>
+</worksheet>
 </file>
</xml_diff>